<commit_message>
Record declared domain expense and three-month website VM budget
</commit_message>
<xml_diff>
--- a/Anjoman accounting - refined.xlsx
+++ b/Anjoman accounting - refined.xlsx
@@ -2,19 +2,20 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="1" r:id="R4a9f4271ec614551"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Monthly report" sheetId="2" r:id="R63cce25b3d4c4c0f"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Project report" sheetId="3" r:id="Rb430486f56924b5f"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Category report" sheetId="4" r:id="R227ce80cdd234da4"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Instructor payments" sheetId="5" r:id="R101d2ef863814210"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Original reconciliation" sheetId="6" r:id="R4bfe70809c4e4662"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Transactions" sheetId="7" r:id="Rd5c3ba573aa249db"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Invoices" sheetId="8" r:id="R858a50cfac1d461f"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Review items" sheetId="9" r:id="R3518424ddf3d4f0f"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Evidence register" sheetId="10" r:id="Re33b57dd606547a8"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Telegram messages" sheetId="11" r:id="R172e6d085a944565"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Original records" sheetId="12" r:id="Rae202dfdac2b4cb6"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Methodology" sheetId="13" r:id="R81e80365f50b4c62"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="1" r:id="Rc1c63eeb9adb4c29"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Monthly report" sheetId="2" r:id="Ra817098cd0ac4f79"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Project report" sheetId="3" r:id="R25d0897a8d5b4bb5"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Category report" sheetId="4" r:id="Redd5d58e56694769"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Instructor payments" sheetId="5" r:id="R961148af21bf4f58"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Original reconciliation" sheetId="6" r:id="R9a0f560a77024b50"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Transactions" sheetId="7" r:id="R0de0e650211f489f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Invoices" sheetId="8" r:id="Rbe296708a34d497a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Review items" sheetId="9" r:id="R29b050f8b1e4485f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Evidence register" sheetId="10" r:id="R2f7091a5aed54313"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Telegram messages" sheetId="11" r:id="R0ae9833c42984309"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Original records" sheetId="12" r:id="R6e89d45c901c4f62"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Methodology" sheetId="13" r:id="R169f3d1f00114fd1"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Website budget" sheetId="14" r:id="R7f4b779fe8c6467e"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -25,12 +26,13 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <x:styleSheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <x:numFmts count="3">
+  <x:numFmts count="4">
     <x:numFmt numFmtId="200" formatCode="yyyy-mm-dd"/>
     <x:numFmt numFmtId="201" formatCode="#,##0.0;(#,##0.0);&quot;-&quot;"/>
     <x:numFmt numFmtId="202" formatCode="#,##0"/>
+    <x:numFmt numFmtId="203" formatCode="0"/>
   </x:numFmts>
-  <x:fonts count="9">
+  <x:fonts count="10">
     <x:font>
       <x:sz val="11"/>
       <x:name val="Carlito"/>
@@ -79,6 +81,11 @@
       <x:color rgb="FFFFFFFF"/>
       <x:name val="Carlito"/>
     </x:font>
+    <x:font>
+      <x:sz val="10"/>
+      <x:color rgb="FF008000"/>
+      <x:name val="Arial"/>
+    </x:font>
   </x:fonts>
   <x:fills count="5">
     <x:fill>
@@ -115,7 +122,7 @@
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="37">
+  <x:cellXfs count="49">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
@@ -197,14 +204,46 @@
     <x:xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment vertical="center" wrapText="1"/>
     </x:xf>
+    <x:xf numFmtId="203" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="200" fontId="4" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="201" fontId="9" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="200" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="203" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="8" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
     <x:xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment wrapText="1"/>
     </x:xf>
     <x:xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment wrapText="1"/>
     </x:xf>
+    <x:xf numFmtId="201" fontId="9" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="201" fontId="4" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
     <x:xf numFmtId="201" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="200" fontId="4" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="203" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="200" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="203" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
     </x:xf>
     <x:xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -474,7 +513,7 @@
       </xdr:xfrm>
       <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R87bb17e6ce894254"/>
+          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R53c92c6846d5404a"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -546,11 +585,23 @@
 </file>
 
 <file path=xl/tables/table13.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="13" name="MethodologyTable" displayName="MethodologyTable" ref="A4:B30" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
-  <x:autoFilter ref="A4:B30"/>
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="13" name="MethodologyTable" displayName="MethodologyTable" ref="A4:B31" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+  <x:autoFilter ref="A4:B31"/>
   <x:tableColumns count="2">
     <x:tableColumn id="1" name="Topic"/>
     <x:tableColumn id="2" name="Policy"/>
+  </x:tableColumns>
+  <x:tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
+</x:table>
+</file>
+
+<file path=xl/tables/table14.xml><?xml version="1.0" encoding="utf-8"?>
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="14" name="WebsitebudgetTable" displayName="WebsitebudgetTable" ref="A4:C13" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+  <x:autoFilter ref="A4:C13"/>
+  <x:tableColumns count="3">
+    <x:tableColumn id="1" name="Measure"/>
+    <x:tableColumn id="2" name="Value"/>
+    <x:tableColumn id="3" name="Basis"/>
   </x:tableColumns>
   <x:tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </x:table>
@@ -572,8 +623,8 @@
 </file>
 
 <file path=xl/tables/table3.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="4" name="ProjectreportTable" displayName="ProjectreportTable" ref="A4:E16" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
-  <x:autoFilter ref="A4:E16"/>
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="4" name="ProjectreportTable" displayName="ProjectreportTable" ref="A4:E17" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+  <x:autoFilter ref="A4:E17"/>
   <x:tableColumns count="5">
     <x:tableColumn id="1" name="Project"/>
     <x:tableColumn id="2" name="Receipts (toman)"/>
@@ -586,8 +637,8 @@
 </file>
 
 <file path=xl/tables/table4.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="5" name="CategoryreportTable" displayName="CategoryreportTable" ref="A4:E17" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
-  <x:autoFilter ref="A4:E17"/>
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="5" name="CategoryreportTable" displayName="CategoryreportTable" ref="A4:E18" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+  <x:autoFilter ref="A4:E18"/>
   <x:tableColumns count="5">
     <x:tableColumn id="1" name="Category"/>
     <x:tableColumn id="2" name="Receipts (toman)"/>
@@ -635,8 +686,8 @@
 </file>
 
 <file path=xl/tables/table7.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="TransactionsTable" displayName="TransactionsTable" ref="A4:Y99" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
-  <x:autoFilter ref="A4:Y99"/>
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="TransactionsTable" displayName="TransactionsTable" ref="A4:Y100" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+  <x:autoFilter ref="A4:Y100"/>
   <x:tableColumns count="25">
     <x:tableColumn id="1" name="ID"/>
     <x:tableColumn id="2" name="Gregorian date"/>
@@ -689,8 +740,8 @@
 </file>
 
 <file path=xl/tables/table9.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="9" name="ReviewitemsTable" displayName="ReviewitemsTable" ref="A4:H19" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
-  <x:autoFilter ref="A4:H19"/>
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="9" name="ReviewitemsTable" displayName="ReviewitemsTable" ref="A4:H20" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+  <x:autoFilter ref="A4:H20"/>
   <x:tableColumns count="8">
     <x:tableColumn id="1" name="Issue ID"/>
     <x:tableColumn id="2" name="Priority"/>
@@ -941,7 +992,7 @@
         <x:v>Supported cash receipts</x:v>
       </x:c>
       <x:c r="B5" s="19" t="n">
-        <x:f>SUM('Transactions'!$W$5:$W$99)</x:f>
+        <x:f>SUM('Transactions'!$W$5:$W$100)</x:f>
         <x:v>112552000</x:v>
       </x:c>
       <x:c r="C5" s="8" t="str">
@@ -953,7 +1004,7 @@
         <x:v>Supported cash payments</x:v>
       </x:c>
       <x:c r="B6" s="19" t="n">
-        <x:f>SUM('Transactions'!$X$5:$X$99)</x:f>
+        <x:f>SUM('Transactions'!$X$5:$X$100)</x:f>
         <x:v>99085195</x:v>
       </x:c>
       <x:c r="C6" s="8" t="str">
@@ -989,7 +1040,7 @@
         <x:v>Receipts awaiting review</x:v>
       </x:c>
       <x:c r="B9" s="19" t="n">
-        <x:f>SUMIFS('Transactions'!$H$5:$H$99,'Transactions'!$N$5:$N$99,"Review",'Transactions'!$E$5:$E$99,"Receipt")</x:f>
+        <x:f>SUMIFS('Transactions'!$H$5:$H$100,'Transactions'!$N$5:$N$100,"Review",'Transactions'!$E$5:$E$100,"Receipt")</x:f>
         <x:v>0</x:v>
       </x:c>
       <x:c r="C9" s="8" t="str">
@@ -1001,8 +1052,8 @@
         <x:v>Payments awaiting review</x:v>
       </x:c>
       <x:c r="B10" s="19" t="n">
-        <x:f>SUMIFS('Transactions'!$H$5:$H$99,'Transactions'!$N$5:$N$99,"Review",'Transactions'!$E$5:$E$99,"Payment")</x:f>
-        <x:v>8334723.9</x:v>
+        <x:f>SUMIFS('Transactions'!$H$5:$H$100,'Transactions'!$N$5:$N$100,"Review",'Transactions'!$E$5:$E$100,"Payment")</x:f>
+        <x:v>11334723.9</x:v>
       </x:c>
       <x:c r="C10" s="8" t="str">
         <x:v>Excluded from supported totals</x:v>
@@ -1013,7 +1064,7 @@
         <x:v>Unclassified amounts awaiting review</x:v>
       </x:c>
       <x:c r="B11" s="19" t="n">
-        <x:f>SUMIFS('Transactions'!$H$5:$H$99,'Transactions'!$N$5:$N$99,"Review",'Transactions'!$E$5:$E$99,"Unknown")</x:f>
+        <x:f>SUMIFS('Transactions'!$H$5:$H$100,'Transactions'!$N$5:$N$100,"Review",'Transactions'!$E$5:$E$100,"Unknown")</x:f>
         <x:v>300000</x:v>
       </x:c>
       <x:c r="C11" s="8" t="str">
@@ -1025,7 +1076,7 @@
         <x:v>Internal transfers</x:v>
       </x:c>
       <x:c r="B12" s="19" t="n">
-        <x:f>SUMIFS('Transactions'!$H$5:$H$99,'Transactions'!$E$5:$E$99,"Internal transfer",'Transactions'!$N$5:$N$99,"Supported")</x:f>
+        <x:f>SUMIFS('Transactions'!$H$5:$H$100,'Transactions'!$E$5:$E$100,"Internal transfer",'Transactions'!$N$5:$N$100,"Supported")</x:f>
         <x:v>0</x:v>
       </x:c>
       <x:c r="C12" s="8" t="str">
@@ -1049,7 +1100,7 @@
         <x:v>Excluded duplicate candidate amounts</x:v>
       </x:c>
       <x:c r="B14" s="19" t="n">
-        <x:f>SUMIFS('Transactions'!$H$5:$H$99,'Transactions'!$N$5:$N$99,"Duplicate")</x:f>
+        <x:f>SUMIFS('Transactions'!$H$5:$H$100,'Transactions'!$N$5:$N$100,"Duplicate")</x:f>
         <x:v>6129375</x:v>
       </x:c>
       <x:c r="C14" s="8" t="str">
@@ -1061,7 +1112,7 @@
         <x:v>Supported transaction count</x:v>
       </x:c>
       <x:c r="B15" s="21" t="n">
-        <x:f>COUNTIFS('Transactions'!$N$5:$N$99,"Supported",'Transactions'!$E$5:$E$99,"Receipt")+COUNTIFS('Transactions'!$N$5:$N$99,"Supported",'Transactions'!$E$5:$E$99,"Payment")</x:f>
+        <x:f>COUNTIFS('Transactions'!$N$5:$N$100,"Supported",'Transactions'!$E$5:$E$100,"Receipt")+COUNTIFS('Transactions'!$N$5:$N$100,"Supported",'Transactions'!$E$5:$E$100,"Payment")</x:f>
         <x:v>66</x:v>
       </x:c>
       <x:c r="C15" s="8" t="str">
@@ -1073,8 +1124,8 @@
         <x:v>Review transaction count</x:v>
       </x:c>
       <x:c r="B16" s="21" t="n">
-        <x:f>COUNTIFS('Transactions'!$N$5:$N$99,"Review")</x:f>
-        <x:v>21</x:v>
+        <x:f>COUNTIFS('Transactions'!$N$5:$N$100,"Review")</x:f>
+        <x:v>22</x:v>
       </x:c>
       <x:c r="C16" s="8" t="str">
         <x:v>Number of ledger records marked Review</x:v>
@@ -1154,7 +1205,7 @@
         <x:v>Former-board handover</x:v>
       </x:c>
       <x:c r="B28" s="30" t="n">
-        <x:f>SUMIFS('Transactions'!$W$5:$W$99,'Transactions'!$L$5:$L$99,"Opening funds")</x:f>
+        <x:f>SUMIFS('Transactions'!$W$5:$W$100,'Transactions'!$L$5:$L$100,"Opening funds")</x:f>
         <x:v>11000000</x:v>
       </x:c>
       <x:c r="C28" s="29" t="str">
@@ -1215,6 +1266,53 @@
       </x:c>
       <x:c r="C34" s="29" t="str">
         <x:v>Zahra Amiri payment; excluded from instructor fees</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="36">
+      <x:c r="A36" s="27" t="str">
+        <x:v>Association website</x:v>
+      </x:c>
+      <x:c r="B36" s="27" t="str">
+        <x:v>Amount (toman)</x:v>
+      </x:c>
+      <x:c r="C36" s="27" t="str">
+        <x:v>Separate from supported cash</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="37" ht="15" hidden="0" customHeight="1">
+      <x:c r="A37" s="29" t="str">
+        <x:v>Declared domain purchase</x:v>
+      </x:c>
+      <x:c r="B37" s="30" t="n">
+        <x:f>'Website budget'!B5</x:f>
+        <x:v>3000000</x:v>
+      </x:c>
+      <x:c r="C37" s="29" t="str">
+        <x:v>Date and funding unconfirmed; included in Review only</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="38" ht="15" hidden="0" customHeight="1">
+      <x:c r="A38" s="29" t="str">
+        <x:v>Three-month VM budget</x:v>
+      </x:c>
+      <x:c r="B38" s="30" t="n">
+        <x:f>'Website budget'!B11</x:f>
+        <x:v>6030048</x:v>
+      </x:c>
+      <x:c r="C38" s="29" t="str">
+        <x:v>92-day estimate; no actual VM payment recorded</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="39" ht="15" hidden="0" customHeight="1">
+      <x:c r="A39" s="29" t="str">
+        <x:v>Combined website budget</x:v>
+      </x:c>
+      <x:c r="B39" s="30" t="n">
+        <x:f>'Website budget'!B12</x:f>
+        <x:v>9030048</x:v>
+      </x:c>
+      <x:c r="C39" s="29" t="str">
+        <x:v>Domain plus VM estimate; not a paid total</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -1224,7 +1322,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rc9ed71cc8aab4345"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Raeb11c1c657f45f7"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -1250,45 +1348,45 @@
   </x:cols>
   <x:sheetData>
     <x:row r="1" ht="15" hidden="0" customHeight="1">
-      <x:c r="A1" s="33"/>
-      <x:c r="B1" s="33"/>
-      <x:c r="C1" s="33"/>
-      <x:c r="D1" s="33"/>
-      <x:c r="E1" s="33"/>
-      <x:c r="F1" s="33"/>
-      <x:c r="G1" s="33"/>
-      <x:c r="H1" s="33"/>
-      <x:c r="I1" s="33"/>
-      <x:c r="J1" s="33"/>
-      <x:c r="K1" s="33"/>
+      <x:c r="A1" s="39"/>
+      <x:c r="B1" s="39"/>
+      <x:c r="C1" s="39"/>
+      <x:c r="D1" s="39"/>
+      <x:c r="E1" s="39"/>
+      <x:c r="F1" s="39"/>
+      <x:c r="G1" s="39"/>
+      <x:c r="H1" s="39"/>
+      <x:c r="I1" s="39"/>
+      <x:c r="J1" s="39"/>
+      <x:c r="K1" s="39"/>
     </x:row>
     <x:row r="2" ht="16.799999237060547" hidden="0" customHeight="1">
-      <x:c r="A2" s="34" t="str">
+      <x:c r="A2" s="40" t="str">
         <x:v>Source inventory and extraction coverage</x:v>
       </x:c>
-      <x:c r="B2" s="33"/>
-      <x:c r="C2" s="33"/>
-      <x:c r="D2" s="33"/>
-      <x:c r="E2" s="33"/>
-      <x:c r="F2" s="33"/>
-      <x:c r="G2" s="33"/>
-      <x:c r="H2" s="33"/>
-      <x:c r="I2" s="33"/>
-      <x:c r="J2" s="33"/>
-      <x:c r="K2" s="33"/>
+      <x:c r="B2" s="39"/>
+      <x:c r="C2" s="39"/>
+      <x:c r="D2" s="39"/>
+      <x:c r="E2" s="39"/>
+      <x:c r="F2" s="39"/>
+      <x:c r="G2" s="39"/>
+      <x:c r="H2" s="39"/>
+      <x:c r="I2" s="39"/>
+      <x:c r="J2" s="39"/>
+      <x:c r="K2" s="39"/>
     </x:row>
     <x:row r="3" ht="15" hidden="0" customHeight="1">
-      <x:c r="A3" s="33"/>
-      <x:c r="B3" s="33"/>
-      <x:c r="C3" s="33"/>
-      <x:c r="D3" s="33"/>
-      <x:c r="E3" s="33"/>
-      <x:c r="F3" s="33"/>
-      <x:c r="G3" s="33"/>
-      <x:c r="H3" s="33"/>
-      <x:c r="I3" s="33"/>
-      <x:c r="J3" s="33"/>
-      <x:c r="K3" s="33"/>
+      <x:c r="A3" s="39"/>
+      <x:c r="B3" s="39"/>
+      <x:c r="C3" s="39"/>
+      <x:c r="D3" s="39"/>
+      <x:c r="E3" s="39"/>
+      <x:c r="F3" s="39"/>
+      <x:c r="G3" s="39"/>
+      <x:c r="H3" s="39"/>
+      <x:c r="I3" s="39"/>
+      <x:c r="J3" s="39"/>
+      <x:c r="K3" s="39"/>
     </x:row>
     <x:row r="4" ht="15" hidden="0" customHeight="1">
       <x:c r="A4" s="7" t="str">
@@ -3897,7 +3995,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R802189b79e394a7a"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rbb033ae8a9dc4ec5"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -3919,33 +4017,33 @@
   </x:cols>
   <x:sheetData>
     <x:row r="1" ht="15" hidden="0" customHeight="1">
-      <x:c r="A1" s="33"/>
-      <x:c r="B1" s="33"/>
-      <x:c r="C1" s="33"/>
-      <x:c r="D1" s="33"/>
-      <x:c r="E1" s="33"/>
-      <x:c r="F1" s="33"/>
-      <x:c r="G1" s="33"/>
+      <x:c r="A1" s="39"/>
+      <x:c r="B1" s="39"/>
+      <x:c r="C1" s="39"/>
+      <x:c r="D1" s="39"/>
+      <x:c r="E1" s="39"/>
+      <x:c r="F1" s="39"/>
+      <x:c r="G1" s="39"/>
     </x:row>
     <x:row r="2" ht="16.799999237060547" hidden="0" customHeight="1">
-      <x:c r="A2" s="34" t="str">
+      <x:c r="A2" s="40" t="str">
         <x:v>Telegram source messages | replies and attachments preserved</x:v>
       </x:c>
-      <x:c r="B2" s="33"/>
-      <x:c r="C2" s="33"/>
-      <x:c r="D2" s="33"/>
-      <x:c r="E2" s="33"/>
-      <x:c r="F2" s="33"/>
-      <x:c r="G2" s="33"/>
+      <x:c r="B2" s="39"/>
+      <x:c r="C2" s="39"/>
+      <x:c r="D2" s="39"/>
+      <x:c r="E2" s="39"/>
+      <x:c r="F2" s="39"/>
+      <x:c r="G2" s="39"/>
     </x:row>
     <x:row r="3" ht="15" hidden="0" customHeight="1">
-      <x:c r="A3" s="33"/>
-      <x:c r="B3" s="33"/>
-      <x:c r="C3" s="33"/>
-      <x:c r="D3" s="33"/>
-      <x:c r="E3" s="33"/>
-      <x:c r="F3" s="33"/>
-      <x:c r="G3" s="33"/>
+      <x:c r="A3" s="39"/>
+      <x:c r="B3" s="39"/>
+      <x:c r="C3" s="39"/>
+      <x:c r="D3" s="39"/>
+      <x:c r="E3" s="39"/>
+      <x:c r="F3" s="39"/>
+      <x:c r="G3" s="39"/>
     </x:row>
     <x:row r="4" ht="15" hidden="0" customHeight="1">
       <x:c r="A4" s="7" t="str">
@@ -7571,7 +7669,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R5f60271f93344373"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R5c0ae5c88bb348bd"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -7591,27 +7689,27 @@
   </x:cols>
   <x:sheetData>
     <x:row r="1" ht="15" hidden="0" customHeight="1">
-      <x:c r="A1" s="33"/>
-      <x:c r="B1" s="33"/>
-      <x:c r="C1" s="33"/>
-      <x:c r="D1" s="33"/>
-      <x:c r="E1" s="33"/>
+      <x:c r="A1" s="39"/>
+      <x:c r="B1" s="39"/>
+      <x:c r="C1" s="39"/>
+      <x:c r="D1" s="39"/>
+      <x:c r="E1" s="39"/>
     </x:row>
     <x:row r="2" ht="16.799999237060547" hidden="0" customHeight="1">
-      <x:c r="A2" s="34" t="str">
+      <x:c r="A2" s="40" t="str">
         <x:v>Original workbook cells | unchanged source snapshots</x:v>
       </x:c>
-      <x:c r="B2" s="33"/>
-      <x:c r="C2" s="33"/>
-      <x:c r="D2" s="33"/>
-      <x:c r="E2" s="33"/>
+      <x:c r="B2" s="39"/>
+      <x:c r="C2" s="39"/>
+      <x:c r="D2" s="39"/>
+      <x:c r="E2" s="39"/>
     </x:row>
     <x:row r="3" ht="15" hidden="0" customHeight="1">
-      <x:c r="A3" s="33"/>
-      <x:c r="B3" s="33"/>
-      <x:c r="C3" s="33"/>
-      <x:c r="D3" s="33"/>
-      <x:c r="E3" s="33"/>
+      <x:c r="A3" s="39"/>
+      <x:c r="B3" s="39"/>
+      <x:c r="C3" s="39"/>
+      <x:c r="D3" s="39"/>
+      <x:c r="E3" s="39"/>
     </x:row>
     <x:row r="4" ht="15" hidden="0" customHeight="1">
       <x:c r="A4" s="7" t="str">
@@ -53440,7 +53538,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R729c94d5ac7a42bc"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R5a32414ed50c48cc"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -53457,18 +53555,18 @@
   </x:cols>
   <x:sheetData>
     <x:row r="1" ht="15" hidden="0" customHeight="1">
-      <x:c r="A1" s="33"/>
-      <x:c r="B1" s="33"/>
+      <x:c r="A1" s="39"/>
+      <x:c r="B1" s="39"/>
     </x:row>
     <x:row r="2" ht="16.799999237060547" hidden="0" customHeight="1">
-      <x:c r="A2" s="34" t="str">
+      <x:c r="A2" s="40" t="str">
         <x:v>Accounting basis, definitions and refresh instructions</x:v>
       </x:c>
-      <x:c r="B2" s="33"/>
+      <x:c r="B2" s="39"/>
     </x:row>
     <x:row r="3" ht="15" hidden="0" customHeight="1">
-      <x:c r="A3" s="33"/>
-      <x:c r="B3" s="33"/>
+      <x:c r="A3" s="39"/>
+      <x:c r="B3" s="39"/>
     </x:row>
     <x:row r="4" ht="15" hidden="0" customHeight="1">
       <x:c r="A4" s="7" t="str">
@@ -53684,6 +53782,14 @@
       </x:c>
       <x:c r="B30" s="31" t="str">
         <x:v>User-confirmation revision: all recipts/ images are association expenses. Provisional transfers and the photographed invoice are treated as settled only on explicit user attestation; their original source limitations remain visible. The folder duplicate is retained and excluded. Five Summer School 1405 payments are identified; the sixth is not inferred.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="31" ht="24" hidden="0" customHeight="1">
+      <x:c r="A31" s="31" t="str">
+        <x:v>Policy 13</x:v>
+      </x:c>
+      <x:c r="B31" s="31" t="str">
+        <x:v>Website costs: the domain is a user-declared 3,000,000 toman expense with unknown purchase date and funding source, held outside cutoff supported cash totals. The VM is a 92-day budget at 655,440 rial per day; projections are not actual payments.</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -53692,7 +53798,328 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R00da56e4d26f4d9a"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R96fbe383ba93417b"/>
+  </x:tableParts>
+</x:worksheet>
+</file>
+
+<file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
+<x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <x:sheetPr>
+    <x:tabColor rgb="FFEDF2F7"/>
+  </x:sheetPr>
+  <x:sheetFormatPr defaultRowHeight="15"/>
+  <x:cols>
+    <x:col min="1" max="1" width="42" hidden="0" customWidth="1"/>
+    <x:col min="2" max="2" width="26" hidden="0" customWidth="1"/>
+    <x:col min="3" max="3" width="105" hidden="0" customWidth="1"/>
+    <x:col min="4" max="4" width="24" hidden="0" customWidth="1"/>
+    <x:col min="5" max="5" width="24" hidden="0" customWidth="1"/>
+  </x:cols>
+  <x:sheetData>
+    <x:row r="1" ht="15" hidden="0" customHeight="1">
+      <x:c r="A1" s="39"/>
+      <x:c r="B1" s="39"/>
+      <x:c r="C1" s="39"/>
+      <x:c r="D1" s="29"/>
+      <x:c r="E1" s="29"/>
+    </x:row>
+    <x:row r="2" ht="16.799999237060547" hidden="0" customHeight="1">
+      <x:c r="A2" s="40" t="str">
+        <x:v>Association website: declared domain expense and VM forecast</x:v>
+      </x:c>
+      <x:c r="B2" s="39"/>
+      <x:c r="C2" s="39"/>
+      <x:c r="D2" s="29"/>
+      <x:c r="E2" s="29"/>
+    </x:row>
+    <x:row r="3" ht="15" hidden="0" customHeight="1">
+      <x:c r="A3" s="39"/>
+      <x:c r="B3" s="39"/>
+      <x:c r="C3" s="39"/>
+      <x:c r="D3" s="29"/>
+      <x:c r="E3" s="29"/>
+    </x:row>
+    <x:row r="4" ht="15" hidden="0" customHeight="1">
+      <x:c r="A4" s="7" t="str">
+        <x:v>Measure</x:v>
+      </x:c>
+      <x:c r="B4" s="7" t="str">
+        <x:v>Value</x:v>
+      </x:c>
+      <x:c r="C4" s="7" t="str">
+        <x:v>Basis</x:v>
+      </x:c>
+      <x:c r="D4" s="29"/>
+      <x:c r="E4" s="29"/>
+    </x:row>
+    <x:row r="5" ht="15" hidden="0" customHeight="1">
+      <x:c r="A5" s="31" t="str">
+        <x:v>Declared domain cost (toman)</x:v>
+      </x:c>
+      <x:c r="B5" s="41" t="n">
+        <x:f>'Transactions'!H100</x:f>
+        <x:v>3000000</x:v>
+      </x:c>
+      <x:c r="C5" s="31" t="str">
+        <x:v>User-declared purchase; date and funding unknown; TX0096 excluded from supported cash</x:v>
+      </x:c>
+      <x:c r="D5" s="29"/>
+      <x:c r="E5" s="29"/>
+    </x:row>
+    <x:row r="6" ht="15" hidden="0" customHeight="1">
+      <x:c r="A6" s="31" t="str">
+        <x:v>Daily VM rate (rial)</x:v>
+      </x:c>
+      <x:c r="B6" s="42" t="n">
+        <x:v>655440</x:v>
+      </x:c>
+      <x:c r="C6" s="31" t="str">
+        <x:v>User quotation; editable rate</x:v>
+      </x:c>
+      <x:c r="D6" s="29"/>
+      <x:c r="E6" s="29"/>
+    </x:row>
+    <x:row r="7" ht="15" hidden="0" customHeight="1">
+      <x:c r="A7" s="31" t="str">
+        <x:v>Daily VM rate (toman)</x:v>
+      </x:c>
+      <x:c r="B7" s="43" t="n">
+        <x:f>IF(ISNUMBER(B6),B6/10,"Unavailable")</x:f>
+        <x:v>65544</x:v>
+      </x:c>
+      <x:c r="C7" s="31" t="str">
+        <x:v>10 rial = 1 toman</x:v>
+      </x:c>
+      <x:c r="D7" s="29"/>
+      <x:c r="E7" s="29"/>
+    </x:row>
+    <x:row r="8" ht="15" hidden="0" customHeight="1">
+      <x:c r="A8" s="31" t="str">
+        <x:v>VM service start</x:v>
+      </x:c>
+      <x:c r="B8" s="44" t="d">
+        <x:v>2026-08-19T00:00:00.000Z</x:v>
+      </x:c>
+      <x:c r="C8" s="31" t="str">
+        <x:v>1405/05/28 at 22:56 Asia/Tehran</x:v>
+      </x:c>
+      <x:c r="D8" s="29"/>
+      <x:c r="E8" s="29"/>
+    </x:row>
+    <x:row r="9" ht="15" hidden="0" customHeight="1">
+      <x:c r="A9" s="31" t="str">
+        <x:v>Three-month horizon end</x:v>
+      </x:c>
+      <x:c r="B9" s="44" t="d">
+        <x:v>2026-11-19T00:00:00.000Z</x:v>
+      </x:c>
+      <x:c r="C9" s="31" t="str">
+        <x:v>1405/08/28 at 22:56 Asia/Tehran</x:v>
+      </x:c>
+      <x:c r="D9" s="29"/>
+      <x:c r="E9" s="29"/>
+    </x:row>
+    <x:row r="10" ht="15" hidden="0" customHeight="1">
+      <x:c r="A10" s="31" t="str">
+        <x:v>Full billable days</x:v>
+      </x:c>
+      <x:c r="B10" s="45" t="n">
+        <x:f>IF(AND(ISNUMBER(B8),ISNUMBER(B9),B9&gt;=B8),B9-B8,"Unavailable")</x:f>
+        <x:v>92</x:v>
+      </x:c>
+      <x:c r="C10" s="31" t="str">
+        <x:v>End minus start; start included, horizon end excluded</x:v>
+      </x:c>
+      <x:c r="D10" s="29"/>
+      <x:c r="E10" s="29"/>
+    </x:row>
+    <x:row r="11" ht="15" hidden="0" customHeight="1">
+      <x:c r="A11" s="31" t="str">
+        <x:v>Three-month VM forecast (toman)</x:v>
+      </x:c>
+      <x:c r="B11" s="43" t="n">
+        <x:f>IF(AND(ISNUMBER(B7),ISNUMBER(B10)),B7*B10,"Unavailable")</x:f>
+        <x:v>6030048</x:v>
+      </x:c>
+      <x:c r="C11" s="31" t="str">
+        <x:v>Budget estimate; no actual VM payments supplied</x:v>
+      </x:c>
+      <x:c r="D11" s="29"/>
+      <x:c r="E11" s="29"/>
+    </x:row>
+    <x:row r="12" ht="15" hidden="0" customHeight="1">
+      <x:c r="A12" s="31" t="str">
+        <x:v>Domain plus VM budget (toman)</x:v>
+      </x:c>
+      <x:c r="B12" s="43" t="n">
+        <x:f>IF(AND(ISNUMBER(B5),ISNUMBER(B11)),B5+B11,"Unavailable")</x:f>
+        <x:v>9030048</x:v>
+      </x:c>
+      <x:c r="C12" s="31" t="str">
+        <x:v>Declared domain cost plus modelled VM cost; not cash paid</x:v>
+      </x:c>
+      <x:c r="D12" s="29"/>
+      <x:c r="E12" s="29"/>
+    </x:row>
+    <x:row r="13" ht="15" hidden="0" customHeight="1">
+      <x:c r="A13" s="31" t="str">
+        <x:v>Actual VM payments</x:v>
+      </x:c>
+      <x:c r="B13" s="31" t="str">
+        <x:f>"Unavailable"</x:f>
+        <x:v>Unavailable</x:v>
+      </x:c>
+      <x:c r="C13" s="31" t="str">
+        <x:v>Unknown; excluded from supported payments</x:v>
+      </x:c>
+      <x:c r="D13" s="29"/>
+      <x:c r="E13" s="29"/>
+    </x:row>
+    <x:row r="14" ht="15" hidden="0" customHeight="1">
+      <x:c r="A14" s="29"/>
+      <x:c r="B14" s="29"/>
+      <x:c r="C14" s="29"/>
+      <x:c r="D14" s="29"/>
+      <x:c r="E14" s="29"/>
+    </x:row>
+    <x:row r="15" ht="15" hidden="0" customHeight="1">
+      <x:c r="A15" s="29"/>
+      <x:c r="B15" s="29"/>
+      <x:c r="C15" s="29"/>
+      <x:c r="D15" s="29"/>
+      <x:c r="E15" s="29"/>
+    </x:row>
+    <x:row r="16" ht="15" hidden="0" customHeight="1">
+      <x:c r="A16" s="29"/>
+      <x:c r="B16" s="29"/>
+      <x:c r="C16" s="29"/>
+      <x:c r="D16" s="29"/>
+      <x:c r="E16" s="29"/>
+    </x:row>
+    <x:row r="17" ht="15" hidden="0" customHeight="1">
+      <x:c r="A17" s="38" t="str">
+        <x:v>Jalali service interval</x:v>
+      </x:c>
+      <x:c r="B17" s="38" t="str">
+        <x:v>Start date</x:v>
+      </x:c>
+      <x:c r="C17" s="38" t="str">
+        <x:v>End date</x:v>
+      </x:c>
+      <x:c r="D17" s="38" t="str">
+        <x:v>Days</x:v>
+      </x:c>
+      <x:c r="E17" s="38" t="str">
+        <x:v>VM forecast (toman)</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="18" ht="15" hidden="0" customHeight="1">
+      <x:c r="A18" s="29" t="str">
+        <x:v>1405/05/28 to 1405/06/28</x:v>
+      </x:c>
+      <x:c r="B18" s="46" t="n">
+        <x:f>B8</x:f>
+        <x:v>46253</x:v>
+      </x:c>
+      <x:c r="C18" s="46" t="d">
+        <x:v>2026-09-19T00:00:00.000Z</x:v>
+      </x:c>
+      <x:c r="D18" s="47" t="n">
+        <x:f>C18-B18</x:f>
+        <x:v>31</x:v>
+      </x:c>
+      <x:c r="E18" s="30" t="n">
+        <x:f>D18*$B$7</x:f>
+        <x:v>2031864</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="19" ht="15" hidden="0" customHeight="1">
+      <x:c r="A19" s="29" t="str">
+        <x:v>1405/06/28 to 1405/07/28</x:v>
+      </x:c>
+      <x:c r="B19" s="46" t="n">
+        <x:f>C18</x:f>
+        <x:v>46284</x:v>
+      </x:c>
+      <x:c r="C19" s="46" t="d">
+        <x:v>2026-10-20T00:00:00.000Z</x:v>
+      </x:c>
+      <x:c r="D19" s="47" t="n">
+        <x:f>C19-B19</x:f>
+        <x:v>31</x:v>
+      </x:c>
+      <x:c r="E19" s="30" t="n">
+        <x:f>D19*$B$7</x:f>
+        <x:v>2031864</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="20" ht="15" hidden="0" customHeight="1">
+      <x:c r="A20" s="29" t="str">
+        <x:v>1405/07/28 to 1405/08/28</x:v>
+      </x:c>
+      <x:c r="B20" s="46" t="n">
+        <x:f>C19</x:f>
+        <x:v>46315</x:v>
+      </x:c>
+      <x:c r="C20" s="46" t="n">
+        <x:f>B9</x:f>
+        <x:v>46345</x:v>
+      </x:c>
+      <x:c r="D20" s="47" t="n">
+        <x:f>C20-B20</x:f>
+        <x:v>30</x:v>
+      </x:c>
+      <x:c r="E20" s="30" t="n">
+        <x:f>D20*$B$7</x:f>
+        <x:v>1966320</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="21" ht="15" hidden="0" customHeight="1">
+      <x:c r="A21" s="29"/>
+      <x:c r="B21" s="29"/>
+      <x:c r="C21" s="29"/>
+      <x:c r="D21" s="29"/>
+      <x:c r="E21" s="29"/>
+    </x:row>
+    <x:row r="22" ht="15" hidden="0" customHeight="1">
+      <x:c r="A22" s="29"/>
+      <x:c r="B22" s="29"/>
+      <x:c r="C22" s="29"/>
+      <x:c r="D22" s="29"/>
+      <x:c r="E22" s="29"/>
+    </x:row>
+    <x:row r="23">
+      <x:c r="A23" s="29" t="str">
+        <x:v>Fixed-rate scenario only. No tax, fees, credits or downtime assumed. Billing statements are required to establish actual VM costs.</x:v>
+      </x:c>
+      <x:c r="B23" s="29"/>
+      <x:c r="C23" s="29"/>
+      <x:c r="D23" s="29"/>
+      <x:c r="E23" s="29"/>
+    </x:row>
+    <x:row r="24">
+      <x:c r="A24" s="29"/>
+      <x:c r="B24" s="29"/>
+      <x:c r="C24" s="29"/>
+      <x:c r="D24" s="29"/>
+      <x:c r="E24" s="29"/>
+    </x:row>
+    <x:row r="25">
+      <x:c r="A25" s="29"/>
+      <x:c r="B25" s="29"/>
+      <x:c r="C25" s="29"/>
+      <x:c r="D25" s="29"/>
+      <x:c r="E25" s="29"/>
+    </x:row>
+  </x:sheetData>
+  <x:mergeCells>
+    <x:mergeCell ref="A2:C2"/>
+    <x:mergeCell ref="A23:E25"/>
+  </x:mergeCells>
+  <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <x:tableParts count="1">
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rb2cec64cd9f748ce"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -53763,11 +54190,11 @@
         <x:v>1404/04</x:v>
       </x:c>
       <x:c r="B5" s="10" t="n">
-        <x:f>SUMIFS('Transactions'!$W$5:$W$99,'Transactions'!$D$5:$D$99,A5)</x:f>
+        <x:f>SUMIFS('Transactions'!$W$5:$W$100,'Transactions'!$D$5:$D$100,A5)</x:f>
         <x:v>0</x:v>
       </x:c>
       <x:c r="C5" s="10" t="n">
-        <x:f>SUMIFS('Transactions'!$X$5:$X$99,'Transactions'!$D$5:$D$99,A5)</x:f>
+        <x:f>SUMIFS('Transactions'!$X$5:$X$100,'Transactions'!$D$5:$D$100,A5)</x:f>
         <x:v>400000</x:v>
       </x:c>
       <x:c r="D5" s="10" t="n">
@@ -53779,7 +54206,7 @@
         <x:v>-400000</x:v>
       </x:c>
       <x:c r="F5" s="10" t="n">
-        <x:f>SUMIFS('Transactions'!$H$5:$H$99,'Transactions'!$D$5:$D$99,A5,'Transactions'!$N$5:$N$99,"Review")</x:f>
+        <x:f>SUMIFS('Transactions'!$H$5:$H$100,'Transactions'!$D$5:$D$100,A5,'Transactions'!$N$5:$N$100,"Review")</x:f>
         <x:v>0</x:v>
       </x:c>
     </x:row>
@@ -53788,11 +54215,11 @@
         <x:v>1404/05</x:v>
       </x:c>
       <x:c r="B6" s="10" t="n">
-        <x:f>SUMIFS('Transactions'!$W$5:$W$99,'Transactions'!$D$5:$D$99,A6)</x:f>
+        <x:f>SUMIFS('Transactions'!$W$5:$W$100,'Transactions'!$D$5:$D$100,A6)</x:f>
         <x:v>33642000</x:v>
       </x:c>
       <x:c r="C6" s="10" t="n">
-        <x:f>SUMIFS('Transactions'!$X$5:$X$99,'Transactions'!$D$5:$D$99,A6)</x:f>
+        <x:f>SUMIFS('Transactions'!$X$5:$X$100,'Transactions'!$D$5:$D$100,A6)</x:f>
         <x:v>13250900</x:v>
       </x:c>
       <x:c r="D6" s="10" t="n">
@@ -53804,7 +54231,7 @@
         <x:v>19991100</x:v>
       </x:c>
       <x:c r="F6" s="10" t="n">
-        <x:f>SUMIFS('Transactions'!$H$5:$H$99,'Transactions'!$D$5:$D$99,A6,'Transactions'!$N$5:$N$99,"Review")</x:f>
+        <x:f>SUMIFS('Transactions'!$H$5:$H$100,'Transactions'!$D$5:$D$100,A6,'Transactions'!$N$5:$N$100,"Review")</x:f>
         <x:v>400000</x:v>
       </x:c>
     </x:row>
@@ -53813,11 +54240,11 @@
         <x:v>1404/06</x:v>
       </x:c>
       <x:c r="B7" s="10" t="n">
-        <x:f>SUMIFS('Transactions'!$W$5:$W$99,'Transactions'!$D$5:$D$99,A7)</x:f>
+        <x:f>SUMIFS('Transactions'!$W$5:$W$100,'Transactions'!$D$5:$D$100,A7)</x:f>
         <x:v>4920000</x:v>
       </x:c>
       <x:c r="C7" s="10" t="n">
-        <x:f>SUMIFS('Transactions'!$X$5:$X$99,'Transactions'!$D$5:$D$99,A7)</x:f>
+        <x:f>SUMIFS('Transactions'!$X$5:$X$100,'Transactions'!$D$5:$D$100,A7)</x:f>
         <x:v>3155000</x:v>
       </x:c>
       <x:c r="D7" s="10" t="n">
@@ -53829,7 +54256,7 @@
         <x:v>21756100</x:v>
       </x:c>
       <x:c r="F7" s="10" t="n">
-        <x:f>SUMIFS('Transactions'!$H$5:$H$99,'Transactions'!$D$5:$D$99,A7,'Transactions'!$N$5:$N$99,"Review")</x:f>
+        <x:f>SUMIFS('Transactions'!$H$5:$H$100,'Transactions'!$D$5:$D$100,A7,'Transactions'!$N$5:$N$100,"Review")</x:f>
         <x:v>0</x:v>
       </x:c>
     </x:row>
@@ -53838,11 +54265,11 @@
         <x:v>1404/07</x:v>
       </x:c>
       <x:c r="B8" s="10" t="n">
-        <x:f>SUMIFS('Transactions'!$W$5:$W$99,'Transactions'!$D$5:$D$99,A8)</x:f>
+        <x:f>SUMIFS('Transactions'!$W$5:$W$100,'Transactions'!$D$5:$D$100,A8)</x:f>
         <x:v>500000</x:v>
       </x:c>
       <x:c r="C8" s="10" t="n">
-        <x:f>SUMIFS('Transactions'!$X$5:$X$99,'Transactions'!$D$5:$D$99,A8)</x:f>
+        <x:f>SUMIFS('Transactions'!$X$5:$X$100,'Transactions'!$D$5:$D$100,A8)</x:f>
         <x:v>2845225</x:v>
       </x:c>
       <x:c r="D8" s="10" t="n">
@@ -53854,7 +54281,7 @@
         <x:v>19410875</x:v>
       </x:c>
       <x:c r="F8" s="10" t="n">
-        <x:f>SUMIFS('Transactions'!$H$5:$H$99,'Transactions'!$D$5:$D$99,A8,'Transactions'!$N$5:$N$99,"Review")</x:f>
+        <x:f>SUMIFS('Transactions'!$H$5:$H$100,'Transactions'!$D$5:$D$100,A8,'Transactions'!$N$5:$N$100,"Review")</x:f>
         <x:v>0</x:v>
       </x:c>
     </x:row>
@@ -53863,11 +54290,11 @@
         <x:v>1404/08</x:v>
       </x:c>
       <x:c r="B9" s="10" t="n">
-        <x:f>SUMIFS('Transactions'!$W$5:$W$99,'Transactions'!$D$5:$D$99,A9)</x:f>
+        <x:f>SUMIFS('Transactions'!$W$5:$W$100,'Transactions'!$D$5:$D$100,A9)</x:f>
         <x:v>11000000</x:v>
       </x:c>
       <x:c r="C9" s="10" t="n">
-        <x:f>SUMIFS('Transactions'!$X$5:$X$99,'Transactions'!$D$5:$D$99,A9)</x:f>
+        <x:f>SUMIFS('Transactions'!$X$5:$X$100,'Transactions'!$D$5:$D$100,A9)</x:f>
         <x:v>10103700</x:v>
       </x:c>
       <x:c r="D9" s="10" t="n">
@@ -53879,7 +54306,7 @@
         <x:v>20307175</x:v>
       </x:c>
       <x:c r="F9" s="10" t="n">
-        <x:f>SUMIFS('Transactions'!$H$5:$H$99,'Transactions'!$D$5:$D$99,A9,'Transactions'!$N$5:$N$99,"Review")</x:f>
+        <x:f>SUMIFS('Transactions'!$H$5:$H$100,'Transactions'!$D$5:$D$100,A9,'Transactions'!$N$5:$N$100,"Review")</x:f>
         <x:v>313000</x:v>
       </x:c>
     </x:row>
@@ -53888,11 +54315,11 @@
         <x:v>1404/09</x:v>
       </x:c>
       <x:c r="B10" s="10" t="n">
-        <x:f>SUMIFS('Transactions'!$W$5:$W$99,'Transactions'!$D$5:$D$99,A10)</x:f>
+        <x:f>SUMIFS('Transactions'!$W$5:$W$100,'Transactions'!$D$5:$D$100,A10)</x:f>
         <x:v>23000000</x:v>
       </x:c>
       <x:c r="C10" s="10" t="n">
-        <x:f>SUMIFS('Transactions'!$X$5:$X$99,'Transactions'!$D$5:$D$99,A10)</x:f>
+        <x:f>SUMIFS('Transactions'!$X$5:$X$100,'Transactions'!$D$5:$D$100,A10)</x:f>
         <x:v>1020000</x:v>
       </x:c>
       <x:c r="D10" s="10" t="n">
@@ -53904,7 +54331,7 @@
         <x:v>42287175</x:v>
       </x:c>
       <x:c r="F10" s="10" t="n">
-        <x:f>SUMIFS('Transactions'!$H$5:$H$99,'Transactions'!$D$5:$D$99,A10,'Transactions'!$N$5:$N$99,"Review")</x:f>
+        <x:f>SUMIFS('Transactions'!$H$5:$H$100,'Transactions'!$D$5:$D$100,A10,'Transactions'!$N$5:$N$100,"Review")</x:f>
         <x:v>0</x:v>
       </x:c>
     </x:row>
@@ -53913,11 +54340,11 @@
         <x:v>1404/10</x:v>
       </x:c>
       <x:c r="B11" s="10" t="n">
-        <x:f>SUMIFS('Transactions'!$W$5:$W$99,'Transactions'!$D$5:$D$99,A11)</x:f>
+        <x:f>SUMIFS('Transactions'!$W$5:$W$100,'Transactions'!$D$5:$D$100,A11)</x:f>
         <x:v>16490000</x:v>
       </x:c>
       <x:c r="C11" s="10" t="n">
-        <x:f>SUMIFS('Transactions'!$X$5:$X$99,'Transactions'!$D$5:$D$99,A11)</x:f>
+        <x:f>SUMIFS('Transactions'!$X$5:$X$100,'Transactions'!$D$5:$D$100,A11)</x:f>
         <x:v>2317000</x:v>
       </x:c>
       <x:c r="D11" s="10" t="n">
@@ -53929,7 +54356,7 @@
         <x:v>56460175</x:v>
       </x:c>
       <x:c r="F11" s="10" t="n">
-        <x:f>SUMIFS('Transactions'!$H$5:$H$99,'Transactions'!$D$5:$D$99,A11,'Transactions'!$N$5:$N$99,"Review")</x:f>
+        <x:f>SUMIFS('Transactions'!$H$5:$H$100,'Transactions'!$D$5:$D$100,A11,'Transactions'!$N$5:$N$100,"Review")</x:f>
         <x:v>7921723.9</x:v>
       </x:c>
     </x:row>
@@ -53938,11 +54365,11 @@
         <x:v>1404/12</x:v>
       </x:c>
       <x:c r="B12" s="10" t="n">
-        <x:f>SUMIFS('Transactions'!$W$5:$W$99,'Transactions'!$D$5:$D$99,A12)</x:f>
+        <x:f>SUMIFS('Transactions'!$W$5:$W$100,'Transactions'!$D$5:$D$100,A12)</x:f>
         <x:v>0</x:v>
       </x:c>
       <x:c r="C12" s="10" t="n">
-        <x:f>SUMIFS('Transactions'!$X$5:$X$99,'Transactions'!$D$5:$D$99,A12)</x:f>
+        <x:f>SUMIFS('Transactions'!$X$5:$X$100,'Transactions'!$D$5:$D$100,A12)</x:f>
         <x:v>1801220</x:v>
       </x:c>
       <x:c r="D12" s="10" t="n">
@@ -53954,7 +54381,7 @@
         <x:v>54658955</x:v>
       </x:c>
       <x:c r="F12" s="10" t="n">
-        <x:f>SUMIFS('Transactions'!$H$5:$H$99,'Transactions'!$D$5:$D$99,A12,'Transactions'!$N$5:$N$99,"Review")</x:f>
+        <x:f>SUMIFS('Transactions'!$H$5:$H$100,'Transactions'!$D$5:$D$100,A12,'Transactions'!$N$5:$N$100,"Review")</x:f>
         <x:v>0</x:v>
       </x:c>
     </x:row>
@@ -53963,11 +54390,11 @@
         <x:v>1405/02</x:v>
       </x:c>
       <x:c r="B13" s="10" t="n">
-        <x:f>SUMIFS('Transactions'!$W$5:$W$99,'Transactions'!$D$5:$D$99,A13)</x:f>
+        <x:f>SUMIFS('Transactions'!$W$5:$W$100,'Transactions'!$D$5:$D$100,A13)</x:f>
         <x:v>0</x:v>
       </x:c>
       <x:c r="C13" s="10" t="n">
-        <x:f>SUMIFS('Transactions'!$X$5:$X$99,'Transactions'!$D$5:$D$99,A13)</x:f>
+        <x:f>SUMIFS('Transactions'!$X$5:$X$100,'Transactions'!$D$5:$D$100,A13)</x:f>
         <x:v>4050000</x:v>
       </x:c>
       <x:c r="D13" s="10" t="n">
@@ -53979,7 +54406,7 @@
         <x:v>50608955</x:v>
       </x:c>
       <x:c r="F13" s="10" t="n">
-        <x:f>SUMIFS('Transactions'!$H$5:$H$99,'Transactions'!$D$5:$D$99,A13,'Transactions'!$N$5:$N$99,"Review")</x:f>
+        <x:f>SUMIFS('Transactions'!$H$5:$H$100,'Transactions'!$D$5:$D$100,A13,'Transactions'!$N$5:$N$100,"Review")</x:f>
         <x:v>0</x:v>
       </x:c>
     </x:row>
@@ -53988,11 +54415,11 @@
         <x:v>1405/05</x:v>
       </x:c>
       <x:c r="B14" s="10" t="n">
-        <x:f>SUMIFS('Transactions'!$W$5:$W$99,'Transactions'!$D$5:$D$99,A14)</x:f>
+        <x:f>SUMIFS('Transactions'!$W$5:$W$100,'Transactions'!$D$5:$D$100,A14)</x:f>
         <x:v>0</x:v>
       </x:c>
       <x:c r="C14" s="10" t="n">
-        <x:f>SUMIFS('Transactions'!$X$5:$X$99,'Transactions'!$D$5:$D$99,A14)</x:f>
+        <x:f>SUMIFS('Transactions'!$X$5:$X$100,'Transactions'!$D$5:$D$100,A14)</x:f>
         <x:v>11217000</x:v>
       </x:c>
       <x:c r="D14" s="10" t="n">
@@ -54004,7 +54431,7 @@
         <x:v>39391955</x:v>
       </x:c>
       <x:c r="F14" s="10" t="n">
-        <x:f>SUMIFS('Transactions'!$H$5:$H$99,'Transactions'!$D$5:$D$99,A14,'Transactions'!$N$5:$N$99,"Review")</x:f>
+        <x:f>SUMIFS('Transactions'!$H$5:$H$100,'Transactions'!$D$5:$D$100,A14,'Transactions'!$N$5:$N$100,"Review")</x:f>
         <x:v>0</x:v>
       </x:c>
     </x:row>
@@ -54013,11 +54440,11 @@
         <x:v>1405/06</x:v>
       </x:c>
       <x:c r="B15" s="10" t="n">
-        <x:f>SUMIFS('Transactions'!$W$5:$W$99,'Transactions'!$D$5:$D$99,A15)</x:f>
+        <x:f>SUMIFS('Transactions'!$W$5:$W$100,'Transactions'!$D$5:$D$100,A15)</x:f>
         <x:v>0</x:v>
       </x:c>
       <x:c r="C15" s="10" t="n">
-        <x:f>SUMIFS('Transactions'!$X$5:$X$99,'Transactions'!$D$5:$D$99,A15)</x:f>
+        <x:f>SUMIFS('Transactions'!$X$5:$X$100,'Transactions'!$D$5:$D$100,A15)</x:f>
         <x:v>9150000</x:v>
       </x:c>
       <x:c r="D15" s="10" t="n">
@@ -54029,7 +54456,7 @@
         <x:v>30241955</x:v>
       </x:c>
       <x:c r="F15" s="10" t="n">
-        <x:f>SUMIFS('Transactions'!$H$5:$H$99,'Transactions'!$D$5:$D$99,A15,'Transactions'!$N$5:$N$99,"Review")</x:f>
+        <x:f>SUMIFS('Transactions'!$H$5:$H$100,'Transactions'!$D$5:$D$100,A15,'Transactions'!$N$5:$N$100,"Review")</x:f>
         <x:v>0</x:v>
       </x:c>
     </x:row>
@@ -54038,11 +54465,11 @@
         <x:v>1405/07</x:v>
       </x:c>
       <x:c r="B16" s="10" t="n">
-        <x:f>SUMIFS('Transactions'!$W$5:$W$99,'Transactions'!$D$5:$D$99,A16)</x:f>
+        <x:f>SUMIFS('Transactions'!$W$5:$W$100,'Transactions'!$D$5:$D$100,A16)</x:f>
         <x:v>23000000</x:v>
       </x:c>
       <x:c r="C16" s="10" t="n">
-        <x:f>SUMIFS('Transactions'!$X$5:$X$99,'Transactions'!$D$5:$D$99,A16)</x:f>
+        <x:f>SUMIFS('Transactions'!$X$5:$X$100,'Transactions'!$D$5:$D$100,A16)</x:f>
         <x:v>39775150</x:v>
       </x:c>
       <x:c r="D16" s="10" t="n">
@@ -54054,7 +54481,7 @@
         <x:v>13466805</x:v>
       </x:c>
       <x:c r="F16" s="10" t="n">
-        <x:f>SUMIFS('Transactions'!$H$5:$H$99,'Transactions'!$D$5:$D$99,A16,'Transactions'!$N$5:$N$99,"Review")</x:f>
+        <x:f>SUMIFS('Transactions'!$H$5:$H$100,'Transactions'!$D$5:$D$100,A16,'Transactions'!$N$5:$N$100,"Review")</x:f>
         <x:v>0</x:v>
       </x:c>
     </x:row>
@@ -54063,11 +54490,11 @@
         <x:v>Undated</x:v>
       </x:c>
       <x:c r="B17" s="10" t="n">
-        <x:f>SUMIFS('Transactions'!$W$5:$W$99,'Transactions'!$D$5:$D$99,A17)</x:f>
+        <x:f>SUMIFS('Transactions'!$W$5:$W$100,'Transactions'!$D$5:$D$100,A17)</x:f>
         <x:v>0</x:v>
       </x:c>
       <x:c r="C17" s="10" t="n">
-        <x:f>SUMIFS('Transactions'!$X$5:$X$99,'Transactions'!$D$5:$D$99,A17)</x:f>
+        <x:f>SUMIFS('Transactions'!$X$5:$X$100,'Transactions'!$D$5:$D$100,A17)</x:f>
         <x:v>0</x:v>
       </x:c>
       <x:c r="D17" s="10" t="n">
@@ -54079,8 +54506,8 @@
         <x:v>13466805</x:v>
       </x:c>
       <x:c r="F17" s="10" t="n">
-        <x:f>SUMIFS('Transactions'!$H$5:$H$99,'Transactions'!$D$5:$D$99,A17,'Transactions'!$N$5:$N$99,"Review")</x:f>
-        <x:v>0</x:v>
+        <x:f>SUMIFS('Transactions'!$H$5:$H$100,'Transactions'!$D$5:$D$100,A17,'Transactions'!$N$5:$N$100,"Review")</x:f>
+        <x:v>3000000</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -54088,9 +54515,9 @@
     <x:mergeCell ref="A2:F2"/>
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R8f0135e3e0584163"/>
+  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R5a417473ff02407a"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R54ba6036f48843ab"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Ra6c81485a7bb4c5e"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -54154,11 +54581,11 @@
         <x:v>Association operations</x:v>
       </x:c>
       <x:c r="B5" s="10" t="n">
-        <x:f>SUMIFS('Transactions'!$W$5:$W$99,'Transactions'!$M$5:$M$99,A5)</x:f>
+        <x:f>SUMIFS('Transactions'!$W$5:$W$100,'Transactions'!$M$5:$M$100,A5)</x:f>
         <x:v>34000000</x:v>
       </x:c>
       <x:c r="C5" s="10" t="n">
-        <x:f>SUMIFS('Transactions'!$X$5:$X$99,'Transactions'!$M$5:$M$99,A5)</x:f>
+        <x:f>SUMIFS('Transactions'!$X$5:$X$100,'Transactions'!$M$5:$M$100,A5)</x:f>
         <x:v>3084700</x:v>
       </x:c>
       <x:c r="D5" s="10" t="n">
@@ -54166,238 +54593,259 @@
         <x:v>30915300</x:v>
       </x:c>
       <x:c r="E5" s="10" t="n">
-        <x:f>SUMIFS('Transactions'!$H$5:$H$99,'Transactions'!$M$5:$M$99,A5,'Transactions'!$N$5:$N$99,"Review")</x:f>
+        <x:f>SUMIFS('Transactions'!$H$5:$H$100,'Transactions'!$M$5:$M$100,A5,'Transactions'!$N$5:$N$100,"Review")</x:f>
         <x:v>13000</x:v>
       </x:c>
     </x:row>
     <x:row r="6" ht="27" customHeight="1">
       <x:c r="A6" s="8" t="str">
-        <x:v>Booths 1404</x:v>
+        <x:v>Association website</x:v>
       </x:c>
       <x:c r="B6" s="10" t="n">
-        <x:f>SUMIFS('Transactions'!$W$5:$W$99,'Transactions'!$M$5:$M$99,A6)</x:f>
+        <x:f>SUMIFS('Transactions'!$W$5:$W$100,'Transactions'!$M$5:$M$100,A6)</x:f>
         <x:v>0</x:v>
       </x:c>
       <x:c r="C6" s="10" t="n">
-        <x:f>SUMIFS('Transactions'!$X$5:$X$99,'Transactions'!$M$5:$M$99,A6)</x:f>
-        <x:v>1995000</x:v>
+        <x:f>SUMIFS('Transactions'!$X$5:$X$100,'Transactions'!$M$5:$M$100,A6)</x:f>
+        <x:v>0</x:v>
       </x:c>
       <x:c r="D6" s="10" t="n">
         <x:f>B6-C6</x:f>
-        <x:v>-1995000</x:v>
+        <x:v>0</x:v>
       </x:c>
       <x:c r="E6" s="10" t="n">
-        <x:f>SUMIFS('Transactions'!$H$5:$H$99,'Transactions'!$M$5:$M$99,A6,'Transactions'!$N$5:$N$99,"Review")</x:f>
-        <x:v>0</x:v>
+        <x:f>SUMIFS('Transactions'!$H$5:$H$100,'Transactions'!$M$5:$M$100,A6,'Transactions'!$N$5:$N$100,"Review")</x:f>
+        <x:v>3000000</x:v>
       </x:c>
     </x:row>
     <x:row r="7" ht="27" customHeight="1">
       <x:c r="A7" s="8" t="str">
-        <x:v>Freshman Party 1404</x:v>
+        <x:v>Booths 1404</x:v>
       </x:c>
       <x:c r="B7" s="10" t="n">
-        <x:f>SUMIFS('Transactions'!$W$5:$W$99,'Transactions'!$M$5:$M$99,A7)</x:f>
+        <x:f>SUMIFS('Transactions'!$W$5:$W$100,'Transactions'!$M$5:$M$100,A7)</x:f>
         <x:v>0</x:v>
       </x:c>
       <x:c r="C7" s="10" t="n">
-        <x:f>SUMIFS('Transactions'!$X$5:$X$99,'Transactions'!$M$5:$M$99,A7)</x:f>
-        <x:v>5774000</x:v>
+        <x:f>SUMIFS('Transactions'!$X$5:$X$100,'Transactions'!$M$5:$M$100,A7)</x:f>
+        <x:v>1995000</x:v>
       </x:c>
       <x:c r="D7" s="10" t="n">
         <x:f>B7-C7</x:f>
-        <x:v>-5774000</x:v>
+        <x:v>-1995000</x:v>
       </x:c>
       <x:c r="E7" s="10" t="n">
-        <x:f>SUMIFS('Transactions'!$H$5:$H$99,'Transactions'!$M$5:$M$99,A7,'Transactions'!$N$5:$N$99,"Review")</x:f>
-        <x:v>300000</x:v>
+        <x:f>SUMIFS('Transactions'!$H$5:$H$100,'Transactions'!$M$5:$M$100,A7,'Transactions'!$N$5:$N$100,"Review")</x:f>
+        <x:v>0</x:v>
       </x:c>
     </x:row>
     <x:row r="8" ht="27" customHeight="1">
       <x:c r="A8" s="8" t="str">
-        <x:v>Intro Event 1404</x:v>
+        <x:v>Freshman Party 1404</x:v>
       </x:c>
       <x:c r="B8" s="10" t="n">
-        <x:f>SUMIFS('Transactions'!$W$5:$W$99,'Transactions'!$M$5:$M$99,A8)</x:f>
-        <x:v>4920000</x:v>
+        <x:f>SUMIFS('Transactions'!$W$5:$W$100,'Transactions'!$M$5:$M$100,A8)</x:f>
+        <x:v>0</x:v>
       </x:c>
       <x:c r="C8" s="10" t="n">
-        <x:f>SUMIFS('Transactions'!$X$5:$X$99,'Transactions'!$M$5:$M$99,A8)</x:f>
-        <x:v>3155000</x:v>
+        <x:f>SUMIFS('Transactions'!$X$5:$X$100,'Transactions'!$M$5:$M$100,A8)</x:f>
+        <x:v>5774000</x:v>
       </x:c>
       <x:c r="D8" s="10" t="n">
         <x:f>B8-C8</x:f>
-        <x:v>1765000</x:v>
+        <x:v>-5774000</x:v>
       </x:c>
       <x:c r="E8" s="10" t="n">
-        <x:f>SUMIFS('Transactions'!$H$5:$H$99,'Transactions'!$M$5:$M$99,A8,'Transactions'!$N$5:$N$99,"Review")</x:f>
-        <x:v>0</x:v>
+        <x:f>SUMIFS('Transactions'!$H$5:$H$100,'Transactions'!$M$5:$M$100,A8,'Transactions'!$N$5:$N$100,"Review")</x:f>
+        <x:v>300000</x:v>
       </x:c>
     </x:row>
     <x:row r="9" ht="27" customHeight="1">
       <x:c r="A9" s="8" t="str">
-        <x:v>Intro Event 1405</x:v>
+        <x:v>Intro Event 1404</x:v>
       </x:c>
       <x:c r="B9" s="10" t="n">
-        <x:f>SUMIFS('Transactions'!$W$5:$W$99,'Transactions'!$M$5:$M$99,A9)</x:f>
-        <x:v>23000000</x:v>
+        <x:f>SUMIFS('Transactions'!$W$5:$W$100,'Transactions'!$M$5:$M$100,A9)</x:f>
+        <x:v>4920000</x:v>
       </x:c>
       <x:c r="C9" s="10" t="n">
-        <x:f>SUMIFS('Transactions'!$X$5:$X$99,'Transactions'!$M$5:$M$99,A9)</x:f>
-        <x:v>5950000</x:v>
+        <x:f>SUMIFS('Transactions'!$X$5:$X$100,'Transactions'!$M$5:$M$100,A9)</x:f>
+        <x:v>3155000</x:v>
       </x:c>
       <x:c r="D9" s="10" t="n">
         <x:f>B9-C9</x:f>
-        <x:v>17050000</x:v>
+        <x:v>1765000</x:v>
       </x:c>
       <x:c r="E9" s="10" t="n">
-        <x:f>SUMIFS('Transactions'!$H$5:$H$99,'Transactions'!$M$5:$M$99,A9,'Transactions'!$N$5:$N$99,"Review")</x:f>
+        <x:f>SUMIFS('Transactions'!$H$5:$H$100,'Transactions'!$M$5:$M$100,A9,'Transactions'!$N$5:$N$100,"Review")</x:f>
         <x:v>0</x:v>
       </x:c>
     </x:row>
     <x:row r="10" ht="27" customHeight="1">
       <x:c r="A10" s="8" t="str">
-        <x:v>Professors assembly Mehr</x:v>
+        <x:v>Intro Event 1405</x:v>
       </x:c>
       <x:c r="B10" s="10" t="n">
-        <x:f>SUMIFS('Transactions'!$W$5:$W$99,'Transactions'!$M$5:$M$99,A10)</x:f>
-        <x:v>500000</x:v>
+        <x:f>SUMIFS('Transactions'!$W$5:$W$100,'Transactions'!$M$5:$M$100,A10)</x:f>
+        <x:v>23000000</x:v>
       </x:c>
       <x:c r="C10" s="10" t="n">
-        <x:f>SUMIFS('Transactions'!$X$5:$X$99,'Transactions'!$M$5:$M$99,A10)</x:f>
-        <x:v>1142375</x:v>
+        <x:f>SUMIFS('Transactions'!$X$5:$X$100,'Transactions'!$M$5:$M$100,A10)</x:f>
+        <x:v>5950000</x:v>
       </x:c>
       <x:c r="D10" s="10" t="n">
         <x:f>B10-C10</x:f>
-        <x:v>-642375</x:v>
+        <x:v>17050000</x:v>
       </x:c>
       <x:c r="E10" s="10" t="n">
-        <x:f>SUMIFS('Transactions'!$H$5:$H$99,'Transactions'!$M$5:$M$99,A10,'Transactions'!$N$5:$N$99,"Review")</x:f>
+        <x:f>SUMIFS('Transactions'!$H$5:$H$100,'Transactions'!$M$5:$M$100,A10,'Transactions'!$N$5:$N$100,"Review")</x:f>
         <x:v>0</x:v>
       </x:c>
     </x:row>
     <x:row r="11" ht="27" customHeight="1">
       <x:c r="A11" s="8" t="str">
-        <x:v>Summer School 1404</x:v>
+        <x:v>Professors assembly Mehr</x:v>
       </x:c>
       <x:c r="B11" s="10" t="n">
-        <x:f>SUMIFS('Transactions'!$W$5:$W$99,'Transactions'!$M$5:$M$99,A11)</x:f>
-        <x:v>33642000</x:v>
+        <x:f>SUMIFS('Transactions'!$W$5:$W$100,'Transactions'!$M$5:$M$100,A11)</x:f>
+        <x:v>500000</x:v>
       </x:c>
       <x:c r="C11" s="10" t="n">
-        <x:f>SUMIFS('Transactions'!$X$5:$X$99,'Transactions'!$M$5:$M$99,A11)</x:f>
-        <x:v>12900900</x:v>
+        <x:f>SUMIFS('Transactions'!$X$5:$X$100,'Transactions'!$M$5:$M$100,A11)</x:f>
+        <x:v>1142375</x:v>
       </x:c>
       <x:c r="D11" s="10" t="n">
         <x:f>B11-C11</x:f>
-        <x:v>20741100</x:v>
+        <x:v>-642375</x:v>
       </x:c>
       <x:c r="E11" s="10" t="n">
-        <x:f>SUMIFS('Transactions'!$H$5:$H$99,'Transactions'!$M$5:$M$99,A11,'Transactions'!$N$5:$N$99,"Review")</x:f>
-        <x:v>400000</x:v>
+        <x:f>SUMIFS('Transactions'!$H$5:$H$100,'Transactions'!$M$5:$M$100,A11,'Transactions'!$N$5:$N$100,"Review")</x:f>
+        <x:v>0</x:v>
       </x:c>
     </x:row>
     <x:row r="12" ht="27" customHeight="1">
       <x:c r="A12" s="8" t="str">
-        <x:v>Summer School 1405</x:v>
+        <x:v>Summer School 1404</x:v>
       </x:c>
       <x:c r="B12" s="10" t="n">
-        <x:f>SUMIFS('Transactions'!$W$5:$W$99,'Transactions'!$M$5:$M$99,A12)</x:f>
-        <x:v>0</x:v>
+        <x:f>SUMIFS('Transactions'!$W$5:$W$100,'Transactions'!$M$5:$M$100,A12)</x:f>
+        <x:v>33642000</x:v>
       </x:c>
       <x:c r="C12" s="10" t="n">
-        <x:f>SUMIFS('Transactions'!$X$5:$X$99,'Transactions'!$M$5:$M$99,A12)</x:f>
-        <x:v>11500000</x:v>
+        <x:f>SUMIFS('Transactions'!$X$5:$X$100,'Transactions'!$M$5:$M$100,A12)</x:f>
+        <x:v>12900900</x:v>
       </x:c>
       <x:c r="D12" s="10" t="n">
         <x:f>B12-C12</x:f>
-        <x:v>-11500000</x:v>
+        <x:v>20741100</x:v>
       </x:c>
       <x:c r="E12" s="10" t="n">
-        <x:f>SUMIFS('Transactions'!$H$5:$H$99,'Transactions'!$M$5:$M$99,A12,'Transactions'!$N$5:$N$99,"Review")</x:f>
-        <x:v>0</x:v>
+        <x:f>SUMIFS('Transactions'!$H$5:$H$100,'Transactions'!$M$5:$M$100,A12,'Transactions'!$N$5:$N$100,"Review")</x:f>
+        <x:v>400000</x:v>
       </x:c>
     </x:row>
     <x:row r="13" ht="27" customHeight="1">
       <x:c r="A13" s="8" t="str">
-        <x:v>Tea &amp; Physics society</x:v>
+        <x:v>Summer School 1405</x:v>
       </x:c>
       <x:c r="B13" s="10" t="n">
-        <x:f>SUMIFS('Transactions'!$W$5:$W$99,'Transactions'!$M$5:$M$99,A13)</x:f>
+        <x:f>SUMIFS('Transactions'!$W$5:$W$100,'Transactions'!$M$5:$M$100,A13)</x:f>
         <x:v>0</x:v>
       </x:c>
       <x:c r="C13" s="10" t="n">
-        <x:f>SUMIFS('Transactions'!$X$5:$X$99,'Transactions'!$M$5:$M$99,A13)</x:f>
-        <x:v>1702850</x:v>
+        <x:f>SUMIFS('Transactions'!$X$5:$X$100,'Transactions'!$M$5:$M$100,A13)</x:f>
+        <x:v>11500000</x:v>
       </x:c>
       <x:c r="D13" s="10" t="n">
         <x:f>B13-C13</x:f>
-        <x:v>-1702850</x:v>
+        <x:v>-11500000</x:v>
       </x:c>
       <x:c r="E13" s="10" t="n">
-        <x:f>SUMIFS('Transactions'!$H$5:$H$99,'Transactions'!$M$5:$M$99,A13,'Transactions'!$N$5:$N$99,"Review")</x:f>
+        <x:f>SUMIFS('Transactions'!$H$5:$H$100,'Transactions'!$M$5:$M$100,A13,'Transactions'!$N$5:$N$100,"Review")</x:f>
         <x:v>0</x:v>
       </x:c>
     </x:row>
     <x:row r="14" ht="27" customHeight="1">
       <x:c r="A14" s="8" t="str">
-        <x:v>Unassigned</x:v>
+        <x:v>Tea &amp; Physics society</x:v>
       </x:c>
       <x:c r="B14" s="10" t="n">
-        <x:f>SUMIFS('Transactions'!$W$5:$W$99,'Transactions'!$M$5:$M$99,A14)</x:f>
+        <x:f>SUMIFS('Transactions'!$W$5:$W$100,'Transactions'!$M$5:$M$100,A14)</x:f>
         <x:v>0</x:v>
       </x:c>
       <x:c r="C14" s="10" t="n">
-        <x:f>SUMIFS('Transactions'!$X$5:$X$99,'Transactions'!$M$5:$M$99,A14)</x:f>
-        <x:v>45513370</x:v>
+        <x:f>SUMIFS('Transactions'!$X$5:$X$100,'Transactions'!$M$5:$M$100,A14)</x:f>
+        <x:v>1702850</x:v>
       </x:c>
       <x:c r="D14" s="10" t="n">
         <x:f>B14-C14</x:f>
-        <x:v>-45513370</x:v>
+        <x:v>-1702850</x:v>
       </x:c>
       <x:c r="E14" s="10" t="n">
-        <x:f>SUMIFS('Transactions'!$H$5:$H$99,'Transactions'!$M$5:$M$99,A14,'Transactions'!$N$5:$N$99,"Review")</x:f>
+        <x:f>SUMIFS('Transactions'!$H$5:$H$100,'Transactions'!$M$5:$M$100,A14,'Transactions'!$N$5:$N$100,"Review")</x:f>
         <x:v>0</x:v>
       </x:c>
     </x:row>
     <x:row r="15" ht="27" customHeight="1">
       <x:c r="A15" s="8" t="str">
-        <x:v>Unknown (likely 1405 summer school)</x:v>
+        <x:v>Unassigned</x:v>
       </x:c>
       <x:c r="B15" s="10" t="n">
-        <x:f>SUMIFS('Transactions'!$W$5:$W$99,'Transactions'!$M$5:$M$99,A15)</x:f>
+        <x:f>SUMIFS('Transactions'!$W$5:$W$100,'Transactions'!$M$5:$M$100,A15)</x:f>
         <x:v>0</x:v>
       </x:c>
       <x:c r="C15" s="10" t="n">
-        <x:f>SUMIFS('Transactions'!$X$5:$X$99,'Transactions'!$M$5:$M$99,A15)</x:f>
-        <x:v>0</x:v>
+        <x:f>SUMIFS('Transactions'!$X$5:$X$100,'Transactions'!$M$5:$M$100,A15)</x:f>
+        <x:v>45513370</x:v>
       </x:c>
       <x:c r="D15" s="10" t="n">
         <x:f>B15-C15</x:f>
-        <x:v>0</x:v>
+        <x:v>-45513370</x:v>
       </x:c>
       <x:c r="E15" s="10" t="n">
-        <x:f>SUMIFS('Transactions'!$H$5:$H$99,'Transactions'!$M$5:$M$99,A15,'Transactions'!$N$5:$N$99,"Review")</x:f>
+        <x:f>SUMIFS('Transactions'!$H$5:$H$100,'Transactions'!$M$5:$M$100,A15,'Transactions'!$N$5:$N$100,"Review")</x:f>
         <x:v>0</x:v>
       </x:c>
     </x:row>
     <x:row r="16" ht="27" customHeight="1">
       <x:c r="A16" s="8" t="str">
-        <x:v>Yalda 1404</x:v>
+        <x:v>Unknown (likely 1405 summer school)</x:v>
       </x:c>
       <x:c r="B16" s="10" t="n">
-        <x:f>SUMIFS('Transactions'!$W$5:$W$99,'Transactions'!$M$5:$M$99,A16)</x:f>
-        <x:v>16490000</x:v>
+        <x:f>SUMIFS('Transactions'!$W$5:$W$100,'Transactions'!$M$5:$M$100,A16)</x:f>
+        <x:v>0</x:v>
       </x:c>
       <x:c r="C16" s="10" t="n">
-        <x:f>SUMIFS('Transactions'!$X$5:$X$99,'Transactions'!$M$5:$M$99,A16)</x:f>
-        <x:v>6367000</x:v>
+        <x:f>SUMIFS('Transactions'!$X$5:$X$100,'Transactions'!$M$5:$M$100,A16)</x:f>
+        <x:v>0</x:v>
       </x:c>
       <x:c r="D16" s="10" t="n">
         <x:f>B16-C16</x:f>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="E16" s="10" t="n">
+        <x:f>SUMIFS('Transactions'!$H$5:$H$100,'Transactions'!$M$5:$M$100,A16,'Transactions'!$N$5:$N$100,"Review")</x:f>
+        <x:v>0</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="17" ht="27" customHeight="1">
+      <x:c r="A17" s="8" t="str">
+        <x:v>Yalda 1404</x:v>
+      </x:c>
+      <x:c r="B17" s="10" t="n">
+        <x:f>SUMIFS('Transactions'!$W$5:$W$100,'Transactions'!$M$5:$M$100,A17)</x:f>
+        <x:v>16490000</x:v>
+      </x:c>
+      <x:c r="C17" s="10" t="n">
+        <x:f>SUMIFS('Transactions'!$X$5:$X$100,'Transactions'!$M$5:$M$100,A17)</x:f>
+        <x:v>6367000</x:v>
+      </x:c>
+      <x:c r="D17" s="10" t="n">
+        <x:f>B17-C17</x:f>
         <x:v>10123000</x:v>
       </x:c>
-      <x:c r="E16" s="10" t="n">
-        <x:f>SUMIFS('Transactions'!$H$5:$H$99,'Transactions'!$M$5:$M$99,A16,'Transactions'!$N$5:$N$99,"Review")</x:f>
+      <x:c r="E17" s="10" t="n">
+        <x:f>SUMIFS('Transactions'!$H$5:$H$100,'Transactions'!$M$5:$M$100,A17,'Transactions'!$N$5:$N$100,"Review")</x:f>
         <x:v>7921723.9</x:v>
       </x:c>
     </x:row>
@@ -54407,7 +54855,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R548e1b0b8dbf4a7d"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rdd7d563e0ada4210"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -54471,11 +54919,11 @@
         <x:v>Advertising</x:v>
       </x:c>
       <x:c r="B5" s="10" t="n">
-        <x:f>SUMIFS('Transactions'!$W$5:$W$99,'Transactions'!$L$5:$L$99,A5)</x:f>
+        <x:f>SUMIFS('Transactions'!$W$5:$W$100,'Transactions'!$L$5:$L$100,A5)</x:f>
         <x:v>0</x:v>
       </x:c>
       <x:c r="C5" s="10" t="n">
-        <x:f>SUMIFS('Transactions'!$X$5:$X$99,'Transactions'!$L$5:$L$99,A5)</x:f>
+        <x:f>SUMIFS('Transactions'!$X$5:$X$100,'Transactions'!$L$5:$L$100,A5)</x:f>
         <x:v>400000</x:v>
       </x:c>
       <x:c r="D5" s="10" t="n">
@@ -54483,7 +54931,7 @@
         <x:v>-400000</x:v>
       </x:c>
       <x:c r="E5" s="10" t="n">
-        <x:f>SUMIFS('Transactions'!$H$5:$H$99,'Transactions'!$L$5:$L$99,A5,'Transactions'!$N$5:$N$99,"Review")</x:f>
+        <x:f>SUMIFS('Transactions'!$H$5:$H$100,'Transactions'!$L$5:$L$100,A5,'Transactions'!$N$5:$N$100,"Review")</x:f>
         <x:v>400000</x:v>
       </x:c>
     </x:row>
@@ -54492,11 +54940,11 @@
         <x:v>Bank fees</x:v>
       </x:c>
       <x:c r="B6" s="10" t="n">
-        <x:f>SUMIFS('Transactions'!$W$5:$W$99,'Transactions'!$L$5:$L$99,A6)</x:f>
+        <x:f>SUMIFS('Transactions'!$W$5:$W$100,'Transactions'!$L$5:$L$100,A6)</x:f>
         <x:v>0</x:v>
       </x:c>
       <x:c r="C6" s="10" t="n">
-        <x:f>SUMIFS('Transactions'!$X$5:$X$99,'Transactions'!$L$5:$L$99,A6)</x:f>
+        <x:f>SUMIFS('Transactions'!$X$5:$X$100,'Transactions'!$L$5:$L$100,A6)</x:f>
         <x:v>900</x:v>
       </x:c>
       <x:c r="D6" s="10" t="n">
@@ -54504,7 +54952,7 @@
         <x:v>-900</x:v>
       </x:c>
       <x:c r="E6" s="10" t="n">
-        <x:f>SUMIFS('Transactions'!$H$5:$H$99,'Transactions'!$L$5:$L$99,A6,'Transactions'!$N$5:$N$99,"Review")</x:f>
+        <x:f>SUMIFS('Transactions'!$H$5:$H$100,'Transactions'!$L$5:$L$100,A6,'Transactions'!$N$5:$N$100,"Review")</x:f>
         <x:v>0</x:v>
       </x:c>
     </x:row>
@@ -54513,11 +54961,11 @@
         <x:v>Course fees</x:v>
       </x:c>
       <x:c r="B7" s="10" t="n">
-        <x:f>SUMIFS('Transactions'!$W$5:$W$99,'Transactions'!$L$5:$L$99,A7)</x:f>
+        <x:f>SUMIFS('Transactions'!$W$5:$W$100,'Transactions'!$L$5:$L$100,A7)</x:f>
         <x:v>33642000</x:v>
       </x:c>
       <x:c r="C7" s="10" t="n">
-        <x:f>SUMIFS('Transactions'!$X$5:$X$99,'Transactions'!$L$5:$L$99,A7)</x:f>
+        <x:f>SUMIFS('Transactions'!$X$5:$X$100,'Transactions'!$L$5:$L$100,A7)</x:f>
         <x:v>0</x:v>
       </x:c>
       <x:c r="D7" s="10" t="n">
@@ -54525,7 +54973,7 @@
         <x:v>33642000</x:v>
       </x:c>
       <x:c r="E7" s="10" t="n">
-        <x:f>SUMIFS('Transactions'!$H$5:$H$99,'Transactions'!$L$5:$L$99,A7,'Transactions'!$N$5:$N$99,"Review")</x:f>
+        <x:f>SUMIFS('Transactions'!$H$5:$H$100,'Transactions'!$L$5:$L$100,A7,'Transactions'!$N$5:$N$100,"Review")</x:f>
         <x:v>0</x:v>
       </x:c>
     </x:row>
@@ -54534,11 +54982,11 @@
         <x:v>Donations</x:v>
       </x:c>
       <x:c r="B8" s="10" t="n">
-        <x:f>SUMIFS('Transactions'!$W$5:$W$99,'Transactions'!$L$5:$L$99,A8)</x:f>
+        <x:f>SUMIFS('Transactions'!$W$5:$W$100,'Transactions'!$L$5:$L$100,A8)</x:f>
         <x:v>39990000</x:v>
       </x:c>
       <x:c r="C8" s="10" t="n">
-        <x:f>SUMIFS('Transactions'!$X$5:$X$99,'Transactions'!$L$5:$L$99,A8)</x:f>
+        <x:f>SUMIFS('Transactions'!$X$5:$X$100,'Transactions'!$L$5:$L$100,A8)</x:f>
         <x:v>0</x:v>
       </x:c>
       <x:c r="D8" s="10" t="n">
@@ -54546,7 +54994,7 @@
         <x:v>39990000</x:v>
       </x:c>
       <x:c r="E8" s="10" t="n">
-        <x:f>SUMIFS('Transactions'!$H$5:$H$99,'Transactions'!$L$5:$L$99,A8,'Transactions'!$N$5:$N$99,"Review")</x:f>
+        <x:f>SUMIFS('Transactions'!$H$5:$H$100,'Transactions'!$L$5:$L$100,A8,'Transactions'!$N$5:$N$100,"Review")</x:f>
         <x:v>0</x:v>
       </x:c>
     </x:row>
@@ -54555,11 +55003,11 @@
         <x:v>Equipment</x:v>
       </x:c>
       <x:c r="B9" s="10" t="n">
-        <x:f>SUMIFS('Transactions'!$W$5:$W$99,'Transactions'!$L$5:$L$99,A9)</x:f>
+        <x:f>SUMIFS('Transactions'!$W$5:$W$100,'Transactions'!$L$5:$L$100,A9)</x:f>
         <x:v>0</x:v>
       </x:c>
       <x:c r="C9" s="10" t="n">
-        <x:f>SUMIFS('Transactions'!$X$5:$X$99,'Transactions'!$L$5:$L$99,A9)</x:f>
+        <x:f>SUMIFS('Transactions'!$X$5:$X$100,'Transactions'!$L$5:$L$100,A9)</x:f>
         <x:v>3545000</x:v>
       </x:c>
       <x:c r="D9" s="10" t="n">
@@ -54567,7 +55015,7 @@
         <x:v>-3545000</x:v>
       </x:c>
       <x:c r="E9" s="10" t="n">
-        <x:f>SUMIFS('Transactions'!$H$5:$H$99,'Transactions'!$L$5:$L$99,A9,'Transactions'!$N$5:$N$99,"Review")</x:f>
+        <x:f>SUMIFS('Transactions'!$H$5:$H$100,'Transactions'!$L$5:$L$100,A9,'Transactions'!$N$5:$N$100,"Review")</x:f>
         <x:v>0</x:v>
       </x:c>
     </x:row>
@@ -54576,11 +55024,11 @@
         <x:v>Events</x:v>
       </x:c>
       <x:c r="B10" s="10" t="n">
-        <x:f>SUMIFS('Transactions'!$W$5:$W$99,'Transactions'!$L$5:$L$99,A10)</x:f>
+        <x:f>SUMIFS('Transactions'!$W$5:$W$100,'Transactions'!$L$5:$L$100,A10)</x:f>
         <x:v>27920000</x:v>
       </x:c>
       <x:c r="C10" s="10" t="n">
-        <x:f>SUMIFS('Transactions'!$X$5:$X$99,'Transactions'!$L$5:$L$99,A10)</x:f>
+        <x:f>SUMIFS('Transactions'!$X$5:$X$100,'Transactions'!$L$5:$L$100,A10)</x:f>
         <x:v>20196000</x:v>
       </x:c>
       <x:c r="D10" s="10" t="n">
@@ -54588,7 +55036,7 @@
         <x:v>7724000</x:v>
       </x:c>
       <x:c r="E10" s="10" t="n">
-        <x:f>SUMIFS('Transactions'!$H$5:$H$99,'Transactions'!$L$5:$L$99,A10,'Transactions'!$N$5:$N$99,"Review")</x:f>
+        <x:f>SUMIFS('Transactions'!$H$5:$H$100,'Transactions'!$L$5:$L$100,A10,'Transactions'!$N$5:$N$100,"Review")</x:f>
         <x:v>7921723.9</x:v>
       </x:c>
     </x:row>
@@ -54597,11 +55045,11 @@
         <x:v>Hospitality</x:v>
       </x:c>
       <x:c r="B11" s="10" t="n">
-        <x:f>SUMIFS('Transactions'!$W$5:$W$99,'Transactions'!$L$5:$L$99,A11)</x:f>
+        <x:f>SUMIFS('Transactions'!$W$5:$W$100,'Transactions'!$L$5:$L$100,A11)</x:f>
         <x:v>0</x:v>
       </x:c>
       <x:c r="C11" s="10" t="n">
-        <x:f>SUMIFS('Transactions'!$X$5:$X$99,'Transactions'!$L$5:$L$99,A11)</x:f>
+        <x:f>SUMIFS('Transactions'!$X$5:$X$100,'Transactions'!$L$5:$L$100,A11)</x:f>
         <x:v>12978125</x:v>
       </x:c>
       <x:c r="D11" s="10" t="n">
@@ -54609,7 +55057,7 @@
         <x:v>-12978125</x:v>
       </x:c>
       <x:c r="E11" s="10" t="n">
-        <x:f>SUMIFS('Transactions'!$H$5:$H$99,'Transactions'!$L$5:$L$99,A11,'Transactions'!$N$5:$N$99,"Review")</x:f>
+        <x:f>SUMIFS('Transactions'!$H$5:$H$100,'Transactions'!$L$5:$L$100,A11,'Transactions'!$N$5:$N$100,"Review")</x:f>
         <x:v>0</x:v>
       </x:c>
     </x:row>
@@ -54618,11 +55066,11 @@
         <x:v>Opening funds</x:v>
       </x:c>
       <x:c r="B12" s="10" t="n">
-        <x:f>SUMIFS('Transactions'!$W$5:$W$99,'Transactions'!$L$5:$L$99,A12)</x:f>
+        <x:f>SUMIFS('Transactions'!$W$5:$W$100,'Transactions'!$L$5:$L$100,A12)</x:f>
         <x:v>11000000</x:v>
       </x:c>
       <x:c r="C12" s="10" t="n">
-        <x:f>SUMIFS('Transactions'!$X$5:$X$99,'Transactions'!$L$5:$L$99,A12)</x:f>
+        <x:f>SUMIFS('Transactions'!$X$5:$X$100,'Transactions'!$L$5:$L$100,A12)</x:f>
         <x:v>0</x:v>
       </x:c>
       <x:c r="D12" s="10" t="n">
@@ -54630,7 +55078,7 @@
         <x:v>11000000</x:v>
       </x:c>
       <x:c r="E12" s="10" t="n">
-        <x:f>SUMIFS('Transactions'!$H$5:$H$99,'Transactions'!$L$5:$L$99,A12,'Transactions'!$N$5:$N$99,"Review")</x:f>
+        <x:f>SUMIFS('Transactions'!$H$5:$H$100,'Transactions'!$L$5:$L$100,A12,'Transactions'!$N$5:$N$100,"Review")</x:f>
         <x:v>0</x:v>
       </x:c>
     </x:row>
@@ -54639,11 +55087,11 @@
         <x:v>Printing</x:v>
       </x:c>
       <x:c r="B13" s="10" t="n">
-        <x:f>SUMIFS('Transactions'!$W$5:$W$99,'Transactions'!$L$5:$L$99,A13)</x:f>
+        <x:f>SUMIFS('Transactions'!$W$5:$W$100,'Transactions'!$L$5:$L$100,A13)</x:f>
         <x:v>0</x:v>
       </x:c>
       <x:c r="C13" s="10" t="n">
-        <x:f>SUMIFS('Transactions'!$X$5:$X$99,'Transactions'!$L$5:$L$99,A13)</x:f>
+        <x:f>SUMIFS('Transactions'!$X$5:$X$100,'Transactions'!$L$5:$L$100,A13)</x:f>
         <x:v>193600</x:v>
       </x:c>
       <x:c r="D13" s="10" t="n">
@@ -54651,7 +55099,7 @@
         <x:v>-193600</x:v>
       </x:c>
       <x:c r="E13" s="10" t="n">
-        <x:f>SUMIFS('Transactions'!$H$5:$H$99,'Transactions'!$L$5:$L$99,A13,'Transactions'!$N$5:$N$99,"Review")</x:f>
+        <x:f>SUMIFS('Transactions'!$H$5:$H$100,'Transactions'!$L$5:$L$100,A13,'Transactions'!$N$5:$N$100,"Review")</x:f>
         <x:v>13000</x:v>
       </x:c>
     </x:row>
@@ -54660,11 +55108,11 @@
         <x:v>Supplies</x:v>
       </x:c>
       <x:c r="B14" s="10" t="n">
-        <x:f>SUMIFS('Transactions'!$W$5:$W$99,'Transactions'!$L$5:$L$99,A14)</x:f>
+        <x:f>SUMIFS('Transactions'!$W$5:$W$100,'Transactions'!$L$5:$L$100,A14)</x:f>
         <x:v>0</x:v>
       </x:c>
       <x:c r="C14" s="10" t="n">
-        <x:f>SUMIFS('Transactions'!$X$5:$X$99,'Transactions'!$L$5:$L$99,A14)</x:f>
+        <x:f>SUMIFS('Transactions'!$X$5:$X$100,'Transactions'!$L$5:$L$100,A14)</x:f>
         <x:v>2246100</x:v>
       </x:c>
       <x:c r="D14" s="10" t="n">
@@ -54672,7 +55120,7 @@
         <x:v>-2246100</x:v>
       </x:c>
       <x:c r="E14" s="10" t="n">
-        <x:f>SUMIFS('Transactions'!$H$5:$H$99,'Transactions'!$L$5:$L$99,A14,'Transactions'!$N$5:$N$99,"Review")</x:f>
+        <x:f>SUMIFS('Transactions'!$H$5:$H$100,'Transactions'!$L$5:$L$100,A14,'Transactions'!$N$5:$N$100,"Review")</x:f>
         <x:v>0</x:v>
       </x:c>
     </x:row>
@@ -54681,11 +55129,11 @@
         <x:v>Teaching</x:v>
       </x:c>
       <x:c r="B15" s="10" t="n">
-        <x:f>SUMIFS('Transactions'!$W$5:$W$99,'Transactions'!$L$5:$L$99,A15)</x:f>
+        <x:f>SUMIFS('Transactions'!$W$5:$W$100,'Transactions'!$L$5:$L$100,A15)</x:f>
         <x:v>0</x:v>
       </x:c>
       <x:c r="C15" s="10" t="n">
-        <x:f>SUMIFS('Transactions'!$X$5:$X$99,'Transactions'!$L$5:$L$99,A15)</x:f>
+        <x:f>SUMIFS('Transactions'!$X$5:$X$100,'Transactions'!$L$5:$L$100,A15)</x:f>
         <x:v>24000000</x:v>
       </x:c>
       <x:c r="D15" s="10" t="n">
@@ -54693,7 +55141,7 @@
         <x:v>-24000000</x:v>
       </x:c>
       <x:c r="E15" s="10" t="n">
-        <x:f>SUMIFS('Transactions'!$H$5:$H$99,'Transactions'!$L$5:$L$99,A15,'Transactions'!$N$5:$N$99,"Review")</x:f>
+        <x:f>SUMIFS('Transactions'!$H$5:$H$100,'Transactions'!$L$5:$L$100,A15,'Transactions'!$N$5:$N$100,"Review")</x:f>
         <x:v>0</x:v>
       </x:c>
     </x:row>
@@ -54702,11 +55150,11 @@
         <x:v>Transfers</x:v>
       </x:c>
       <x:c r="B16" s="10" t="n">
-        <x:f>SUMIFS('Transactions'!$W$5:$W$99,'Transactions'!$L$5:$L$99,A16)</x:f>
+        <x:f>SUMIFS('Transactions'!$W$5:$W$100,'Transactions'!$L$5:$L$100,A16)</x:f>
         <x:v>0</x:v>
       </x:c>
       <x:c r="C16" s="10" t="n">
-        <x:f>SUMIFS('Transactions'!$X$5:$X$99,'Transactions'!$L$5:$L$99,A16)</x:f>
+        <x:f>SUMIFS('Transactions'!$X$5:$X$100,'Transactions'!$L$5:$L$100,A16)</x:f>
         <x:v>0</x:v>
       </x:c>
       <x:c r="D16" s="10" t="n">
@@ -54714,7 +55162,7 @@
         <x:v>0</x:v>
       </x:c>
       <x:c r="E16" s="10" t="n">
-        <x:f>SUMIFS('Transactions'!$H$5:$H$99,'Transactions'!$L$5:$L$99,A16,'Transactions'!$N$5:$N$99,"Review")</x:f>
+        <x:f>SUMIFS('Transactions'!$H$5:$H$100,'Transactions'!$L$5:$L$100,A16,'Transactions'!$N$5:$N$100,"Review")</x:f>
         <x:v>0</x:v>
       </x:c>
     </x:row>
@@ -54723,11 +55171,11 @@
         <x:v>Unclassified</x:v>
       </x:c>
       <x:c r="B17" s="10" t="n">
-        <x:f>SUMIFS('Transactions'!$W$5:$W$99,'Transactions'!$L$5:$L$99,A17)</x:f>
+        <x:f>SUMIFS('Transactions'!$W$5:$W$100,'Transactions'!$L$5:$L$100,A17)</x:f>
         <x:v>0</x:v>
       </x:c>
       <x:c r="C17" s="10" t="n">
-        <x:f>SUMIFS('Transactions'!$X$5:$X$99,'Transactions'!$L$5:$L$99,A17)</x:f>
+        <x:f>SUMIFS('Transactions'!$X$5:$X$100,'Transactions'!$L$5:$L$100,A17)</x:f>
         <x:v>35525470</x:v>
       </x:c>
       <x:c r="D17" s="10" t="n">
@@ -54735,8 +55183,29 @@
         <x:v>-35525470</x:v>
       </x:c>
       <x:c r="E17" s="10" t="n">
-        <x:f>SUMIFS('Transactions'!$H$5:$H$99,'Transactions'!$L$5:$L$99,A17,'Transactions'!$N$5:$N$99,"Review")</x:f>
+        <x:f>SUMIFS('Transactions'!$H$5:$H$100,'Transactions'!$L$5:$L$100,A17,'Transactions'!$N$5:$N$100,"Review")</x:f>
         <x:v>300000</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="18" ht="27" customHeight="1">
+      <x:c r="A18" s="8" t="str">
+        <x:v>Website domain</x:v>
+      </x:c>
+      <x:c r="B18" s="10" t="n">
+        <x:f>SUMIFS('Transactions'!$W$5:$W$100,'Transactions'!$L$5:$L$100,A18)</x:f>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="C18" s="10" t="n">
+        <x:f>SUMIFS('Transactions'!$X$5:$X$100,'Transactions'!$L$5:$L$100,A18)</x:f>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="D18" s="10" t="n">
+        <x:f>B18-C18</x:f>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="E18" s="10" t="n">
+        <x:f>SUMIFS('Transactions'!$H$5:$H$100,'Transactions'!$L$5:$L$100,A18,'Transactions'!$N$5:$N$100,"Review")</x:f>
+        <x:v>3000000</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -54745,7 +55214,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R0477bb1193294e00"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R62d2b30e1bc04792"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -54771,45 +55240,45 @@
   </x:cols>
   <x:sheetData>
     <x:row r="1" ht="15" hidden="0" customHeight="1">
-      <x:c r="A1" s="33"/>
-      <x:c r="B1" s="33"/>
-      <x:c r="C1" s="33"/>
-      <x:c r="D1" s="33"/>
-      <x:c r="E1" s="33"/>
-      <x:c r="F1" s="33"/>
-      <x:c r="G1" s="33"/>
-      <x:c r="H1" s="33"/>
-      <x:c r="I1" s="33"/>
-      <x:c r="J1" s="33"/>
-      <x:c r="K1" s="33"/>
+      <x:c r="A1" s="39"/>
+      <x:c r="B1" s="39"/>
+      <x:c r="C1" s="39"/>
+      <x:c r="D1" s="39"/>
+      <x:c r="E1" s="39"/>
+      <x:c r="F1" s="39"/>
+      <x:c r="G1" s="39"/>
+      <x:c r="H1" s="39"/>
+      <x:c r="I1" s="39"/>
+      <x:c r="J1" s="39"/>
+      <x:c r="K1" s="39"/>
     </x:row>
     <x:row r="2" ht="16.799999237060547" hidden="0" customHeight="1">
-      <x:c r="A2" s="34" t="str">
+      <x:c r="A2" s="40" t="str">
         <x:v>Summer School 1405 instructor payments | five of six identified</x:v>
       </x:c>
-      <x:c r="B2" s="33"/>
-      <x:c r="C2" s="33"/>
-      <x:c r="D2" s="33"/>
-      <x:c r="E2" s="33"/>
-      <x:c r="F2" s="33"/>
-      <x:c r="G2" s="33"/>
-      <x:c r="H2" s="33"/>
-      <x:c r="I2" s="33"/>
-      <x:c r="J2" s="33"/>
-      <x:c r="K2" s="33"/>
+      <x:c r="B2" s="39"/>
+      <x:c r="C2" s="39"/>
+      <x:c r="D2" s="39"/>
+      <x:c r="E2" s="39"/>
+      <x:c r="F2" s="39"/>
+      <x:c r="G2" s="39"/>
+      <x:c r="H2" s="39"/>
+      <x:c r="I2" s="39"/>
+      <x:c r="J2" s="39"/>
+      <x:c r="K2" s="39"/>
     </x:row>
     <x:row r="3" ht="15" hidden="0" customHeight="1">
-      <x:c r="A3" s="33"/>
-      <x:c r="B3" s="33"/>
-      <x:c r="C3" s="33"/>
-      <x:c r="D3" s="33"/>
-      <x:c r="E3" s="33"/>
-      <x:c r="F3" s="33"/>
-      <x:c r="G3" s="33"/>
-      <x:c r="H3" s="33"/>
-      <x:c r="I3" s="33"/>
-      <x:c r="J3" s="33"/>
-      <x:c r="K3" s="33"/>
+      <x:c r="A3" s="39"/>
+      <x:c r="B3" s="39"/>
+      <x:c r="C3" s="39"/>
+      <x:c r="D3" s="39"/>
+      <x:c r="E3" s="39"/>
+      <x:c r="F3" s="39"/>
+      <x:c r="G3" s="39"/>
+      <x:c r="H3" s="39"/>
+      <x:c r="I3" s="39"/>
+      <x:c r="J3" s="39"/>
+      <x:c r="K3" s="39"/>
     </x:row>
     <x:row r="4" ht="24" hidden="0" customHeight="1">
       <x:c r="A4" s="7" t="str">
@@ -54865,10 +55334,10 @@
       <x:c r="F5" s="31" t="str">
         <x:v>2026-09-21</x:v>
       </x:c>
-      <x:c r="G5" s="35" t="n">
+      <x:c r="G5" s="43" t="n">
         <x:v>600000</x:v>
       </x:c>
-      <x:c r="H5" s="36" t="str">
+      <x:c r="H5" s="48" t="str">
         <x:v>6104</x:v>
       </x:c>
       <x:c r="I5" s="31" t="str">
@@ -54901,10 +55370,10 @@
       <x:c r="F6" s="31" t="str">
         <x:v>2026-09-21</x:v>
       </x:c>
-      <x:c r="G6" s="35" t="n">
+      <x:c r="G6" s="43" t="n">
         <x:v>1200000</x:v>
       </x:c>
-      <x:c r="H6" s="36" t="str">
+      <x:c r="H6" s="48" t="str">
         <x:v>2692</x:v>
       </x:c>
       <x:c r="I6" s="31" t="str">
@@ -54937,10 +55406,10 @@
       <x:c r="F7" s="31" t="str">
         <x:v>2026-09-21</x:v>
       </x:c>
-      <x:c r="G7" s="35" t="n">
+      <x:c r="G7" s="43" t="n">
         <x:v>2400000</x:v>
       </x:c>
-      <x:c r="H7" s="36" t="str"/>
+      <x:c r="H7" s="48" t="str"/>
       <x:c r="I7" s="31" t="str">
         <x:v>Explicit user confirmation that payment to Alireza was instructor fee for Abolfazl.</x:v>
       </x:c>
@@ -54971,10 +55440,10 @@
       <x:c r="F8" s="31" t="str">
         <x:v>2026-09-23</x:v>
       </x:c>
-      <x:c r="G8" s="35" t="n">
+      <x:c r="G8" s="43" t="n">
         <x:v>4700000</x:v>
       </x:c>
-      <x:c r="H8" s="36" t="str">
+      <x:c r="H8" s="48" t="str">
         <x:v>5740</x:v>
       </x:c>
       <x:c r="I8" s="31" t="str">
@@ -55007,10 +55476,10 @@
       <x:c r="F9" s="31" t="str">
         <x:v>2026-09-23</x:v>
       </x:c>
-      <x:c r="G9" s="35" t="n">
+      <x:c r="G9" s="43" t="n">
         <x:v>2600000</x:v>
       </x:c>
-      <x:c r="H9" s="36" t="str">
+      <x:c r="H9" s="48" t="str">
         <x:v>6676</x:v>
       </x:c>
       <x:c r="I9" s="31" t="str">
@@ -55098,7 +55567,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Ree2b4ec7ce2d4059"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rffbc5b7a559045e6"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -55119,30 +55588,30 @@
   </x:cols>
   <x:sheetData>
     <x:row r="1" ht="15" hidden="0" customHeight="1">
-      <x:c r="A1" s="33"/>
-      <x:c r="B1" s="33"/>
-      <x:c r="C1" s="33"/>
-      <x:c r="D1" s="33"/>
-      <x:c r="E1" s="33"/>
-      <x:c r="F1" s="33"/>
+      <x:c r="A1" s="39"/>
+      <x:c r="B1" s="39"/>
+      <x:c r="C1" s="39"/>
+      <x:c r="D1" s="39"/>
+      <x:c r="E1" s="39"/>
+      <x:c r="F1" s="39"/>
     </x:row>
     <x:row r="2" ht="16.799999237060547" hidden="0" customHeight="1">
-      <x:c r="A2" s="34" t="str">
+      <x:c r="A2" s="40" t="str">
         <x:v>Original ledger rows reconciled to evidence</x:v>
       </x:c>
-      <x:c r="B2" s="33"/>
-      <x:c r="C2" s="33"/>
-      <x:c r="D2" s="33"/>
-      <x:c r="E2" s="33"/>
-      <x:c r="F2" s="33"/>
+      <x:c r="B2" s="39"/>
+      <x:c r="C2" s="39"/>
+      <x:c r="D2" s="39"/>
+      <x:c r="E2" s="39"/>
+      <x:c r="F2" s="39"/>
     </x:row>
     <x:row r="3" ht="15" hidden="0" customHeight="1">
-      <x:c r="A3" s="33"/>
-      <x:c r="B3" s="33"/>
-      <x:c r="C3" s="33"/>
-      <x:c r="D3" s="33"/>
-      <x:c r="E3" s="33"/>
-      <x:c r="F3" s="33"/>
+      <x:c r="A3" s="39"/>
+      <x:c r="B3" s="39"/>
+      <x:c r="C3" s="39"/>
+      <x:c r="D3" s="39"/>
+      <x:c r="E3" s="39"/>
+      <x:c r="F3" s="39"/>
     </x:row>
     <x:row r="4" ht="15" hidden="0" customHeight="1">
       <x:c r="A4" s="7" t="str">
@@ -55171,7 +55640,7 @@
       <x:c r="B5" s="31" t="str">
         <x:v>B3</x:v>
       </x:c>
-      <x:c r="C5" s="35" t="n">
+      <x:c r="C5" s="43" t="n">
         <x:v>33642000</x:v>
       </x:c>
       <x:c r="D5" s="31" t="str">
@@ -55191,7 +55660,7 @@
       <x:c r="B6" s="31" t="str">
         <x:v>D2</x:v>
       </x:c>
-      <x:c r="C6" s="35" t="n">
+      <x:c r="C6" s="43" t="n">
         <x:v>3500000</x:v>
       </x:c>
       <x:c r="D6" s="31" t="str">
@@ -55211,7 +55680,7 @@
       <x:c r="B7" s="31" t="str">
         <x:v>D3</x:v>
       </x:c>
-      <x:c r="C7" s="35" t="n">
+      <x:c r="C7" s="43" t="n">
         <x:v>3000000</x:v>
       </x:c>
       <x:c r="D7" s="31" t="str">
@@ -55231,7 +55700,7 @@
       <x:c r="B8" s="31" t="str">
         <x:v>D4</x:v>
       </x:c>
-      <x:c r="C8" s="35" t="n">
+      <x:c r="C8" s="43" t="n">
         <x:v>3700000</x:v>
       </x:c>
       <x:c r="D8" s="31" t="str">
@@ -55251,7 +55720,7 @@
       <x:c r="B9" s="31" t="str">
         <x:v>D5</x:v>
       </x:c>
-      <x:c r="C9" s="35" t="n">
+      <x:c r="C9" s="43" t="n">
         <x:v>500000</x:v>
       </x:c>
       <x:c r="D9" s="31" t="str">
@@ -55271,7 +55740,7 @@
       <x:c r="B10" s="31" t="str">
         <x:v>D6</x:v>
       </x:c>
-      <x:c r="C10" s="35" t="n">
+      <x:c r="C10" s="43" t="n">
         <x:v>600000</x:v>
       </x:c>
       <x:c r="D10" s="31" t="str">
@@ -55291,7 +55760,7 @@
       <x:c r="B11" s="31" t="str">
         <x:v>D7</x:v>
       </x:c>
-      <x:c r="C11" s="35" t="n">
+      <x:c r="C11" s="43" t="n">
         <x:v>600000</x:v>
       </x:c>
       <x:c r="D11" s="31" t="str">
@@ -55311,7 +55780,7 @@
       <x:c r="B12" s="31" t="str">
         <x:v>D8</x:v>
       </x:c>
-      <x:c r="C12" s="35" t="n">
+      <x:c r="C12" s="43" t="n">
         <x:v>300000</x:v>
       </x:c>
       <x:c r="D12" s="31" t="str">
@@ -55331,7 +55800,7 @@
       <x:c r="B13" s="31" t="str">
         <x:v>D9</x:v>
       </x:c>
-      <x:c r="C13" s="35" t="n">
+      <x:c r="C13" s="43" t="n">
         <x:v>400000</x:v>
       </x:c>
       <x:c r="D13" s="31" t="str">
@@ -55351,7 +55820,7 @@
       <x:c r="B14" s="31" t="str">
         <x:v>D10</x:v>
       </x:c>
-      <x:c r="C14" s="35" t="n">
+      <x:c r="C14" s="43" t="n">
         <x:v>300000</x:v>
       </x:c>
       <x:c r="D14" s="31" t="str">
@@ -55371,7 +55840,7 @@
       <x:c r="B15" s="31" t="str">
         <x:v>D11</x:v>
       </x:c>
-      <x:c r="C15" s="35" t="n">
+      <x:c r="C15" s="43" t="n">
         <x:v>750000</x:v>
       </x:c>
       <x:c r="D15" s="31" t="str">
@@ -55391,7 +55860,7 @@
       <x:c r="B16" s="31" t="str">
         <x:v>D12</x:v>
       </x:c>
-      <x:c r="C16" s="35" t="n">
+      <x:c r="C16" s="43" t="n">
         <x:v>400000</x:v>
       </x:c>
       <x:c r="D16" s="31" t="str">
@@ -55411,7 +55880,7 @@
       <x:c r="B17" s="31" t="str">
         <x:v>B15</x:v>
       </x:c>
-      <x:c r="C17" s="35" t="n">
+      <x:c r="C17" s="43" t="n">
         <x:v>4920000</x:v>
       </x:c>
       <x:c r="D17" s="31" t="str">
@@ -55431,7 +55900,7 @@
       <x:c r="B18" s="31" t="str">
         <x:v>D15</x:v>
       </x:c>
-      <x:c r="C18" s="35" t="n">
+      <x:c r="C18" s="43" t="n">
         <x:v>100000</x:v>
       </x:c>
       <x:c r="D18" s="31" t="str">
@@ -55451,7 +55920,7 @@
       <x:c r="B19" s="31" t="str">
         <x:v>D16</x:v>
       </x:c>
-      <x:c r="C19" s="35" t="n">
+      <x:c r="C19" s="43" t="n">
         <x:v>2866000</x:v>
       </x:c>
       <x:c r="D19" s="31" t="str">
@@ -55471,7 +55940,7 @@
       <x:c r="B20" s="31" t="str">
         <x:v>D17</x:v>
       </x:c>
-      <x:c r="C20" s="35" t="n">
+      <x:c r="C20" s="43" t="n">
         <x:v>189000</x:v>
       </x:c>
       <x:c r="D20" s="31" t="str">
@@ -55491,7 +55960,7 @@
       <x:c r="B21" s="31" t="str">
         <x:v>B19</x:v>
       </x:c>
-      <x:c r="C21" s="35" t="n">
+      <x:c r="C21" s="43" t="n">
         <x:v>500000</x:v>
       </x:c>
       <x:c r="D21" s="31" t="str">
@@ -55511,7 +55980,7 @@
       <x:c r="B22" s="31" t="str">
         <x:v>D19</x:v>
       </x:c>
-      <x:c r="C22" s="35" t="n">
+      <x:c r="C22" s="43" t="n">
         <x:v>90000</x:v>
       </x:c>
       <x:c r="D22" s="31" t="str">
@@ -55531,7 +56000,7 @@
       <x:c r="B23" s="31" t="str">
         <x:v>D20</x:v>
       </x:c>
-      <x:c r="C23" s="35" t="n">
+      <x:c r="C23" s="43" t="n">
         <x:v>1052375</x:v>
       </x:c>
       <x:c r="D23" s="31" t="str">
@@ -55551,7 +56020,7 @@
       <x:c r="B24" s="31" t="str">
         <x:v>D21</x:v>
       </x:c>
-      <x:c r="C24" s="35" t="n">
+      <x:c r="C24" s="43" t="n">
         <x:v>790000</x:v>
       </x:c>
       <x:c r="D24" s="31" t="str">
@@ -55571,7 +56040,7 @@
       <x:c r="B25" s="31" t="str">
         <x:v>D22</x:v>
       </x:c>
-      <x:c r="C25" s="35" t="n">
+      <x:c r="C25" s="43" t="n">
         <x:v>912850</x:v>
       </x:c>
       <x:c r="D25" s="31" t="str">
@@ -55591,7 +56060,7 @@
       <x:c r="B26" s="31" t="str">
         <x:v>D23</x:v>
       </x:c>
-      <x:c r="C26" s="35" t="n">
+      <x:c r="C26" s="43" t="n">
         <x:v>1052375</x:v>
       </x:c>
       <x:c r="D26" s="31" t="str">
@@ -55611,7 +56080,7 @@
       <x:c r="B27" s="31" t="str">
         <x:v>B25</x:v>
       </x:c>
-      <x:c r="C27" s="35" t="n">
+      <x:c r="C27" s="43" t="n">
         <x:v>11000000</x:v>
       </x:c>
       <x:c r="D27" s="31" t="str">
@@ -55631,7 +56100,7 @@
       <x:c r="B28" s="31" t="str">
         <x:v>D25</x:v>
       </x:c>
-      <x:c r="C28" s="35" t="n">
+      <x:c r="C28" s="43" t="n">
         <x:v>725000</x:v>
       </x:c>
       <x:c r="D28" s="31" t="str">
@@ -55651,7 +56120,7 @@
       <x:c r="B29" s="31" t="str">
         <x:v>D26</x:v>
       </x:c>
-      <x:c r="C29" s="35" t="n">
+      <x:c r="C29" s="43" t="n">
         <x:v>120000</x:v>
       </x:c>
       <x:c r="D29" s="31" t="str">
@@ -55671,7 +56140,7 @@
       <x:c r="B30" s="31" t="str">
         <x:v>D27</x:v>
       </x:c>
-      <x:c r="C30" s="35" t="n">
+      <x:c r="C30" s="43" t="n">
         <x:v>1310000</x:v>
       </x:c>
       <x:c r="D30" s="31" t="str">
@@ -55691,7 +56160,7 @@
       <x:c r="B31" s="31" t="str">
         <x:v>D28</x:v>
       </x:c>
-      <x:c r="C31" s="35" t="n">
+      <x:c r="C31" s="43" t="n">
         <x:v>4344000</x:v>
       </x:c>
       <x:c r="D31" s="31" t="str">
@@ -55711,7 +56180,7 @@
       <x:c r="B32" s="31" t="str">
         <x:v>D29</x:v>
       </x:c>
-      <x:c r="C32" s="35" t="n">
+      <x:c r="C32" s="43" t="n">
         <x:v>300000</x:v>
       </x:c>
       <x:c r="D32" s="31" t="str">
@@ -55731,7 +56200,7 @@
       <x:c r="B33" s="31" t="str">
         <x:v>D30</x:v>
       </x:c>
-      <x:c r="C33" s="35" t="n">
+      <x:c r="C33" s="43" t="n">
         <x:v>70000</x:v>
       </x:c>
       <x:c r="D33" s="31" t="str">
@@ -55751,7 +56220,7 @@
       <x:c r="B34" s="31" t="str">
         <x:v>D31</x:v>
       </x:c>
-      <x:c r="C34" s="35" t="n">
+      <x:c r="C34" s="43" t="n">
         <x:v>310000</x:v>
       </x:c>
       <x:c r="D34" s="31" t="str">
@@ -55771,7 +56240,7 @@
       <x:c r="B35" s="31" t="str">
         <x:v>D32</x:v>
       </x:c>
-      <x:c r="C35" s="35" t="n">
+      <x:c r="C35" s="43" t="n">
         <x:v>1760000</x:v>
       </x:c>
       <x:c r="D35" s="31" t="str">
@@ -55791,7 +56260,7 @@
       <x:c r="B36" s="31" t="str">
         <x:v>D33</x:v>
       </x:c>
-      <x:c r="C36" s="35" t="n">
+      <x:c r="C36" s="43" t="n">
         <x:v>230000</x:v>
       </x:c>
       <x:c r="D36" s="31" t="str">
@@ -55811,7 +56280,7 @@
       <x:c r="B37" s="31" t="str">
         <x:v>D34</x:v>
       </x:c>
-      <x:c r="C37" s="35" t="n">
+      <x:c r="C37" s="43" t="n">
         <x:v>1226100</x:v>
       </x:c>
       <x:c r="D37" s="31" t="str">
@@ -55831,7 +56300,7 @@
       <x:c r="B38" s="31" t="str">
         <x:v>D35</x:v>
       </x:c>
-      <x:c r="C38" s="35" t="n">
+      <x:c r="C38" s="43" t="n">
         <x:v>2300</x:v>
       </x:c>
       <x:c r="D38" s="31" t="str">
@@ -55851,7 +56320,7 @@
       <x:c r="B39" s="31" t="str">
         <x:v>D36</x:v>
       </x:c>
-      <x:c r="C39" s="35" t="n">
+      <x:c r="C39" s="43" t="n">
         <x:v>1300</x:v>
       </x:c>
       <x:c r="D39" s="31" t="str">
@@ -55871,7 +56340,7 @@
       <x:c r="B40" s="31" t="str">
         <x:v>B38</x:v>
       </x:c>
-      <x:c r="C40" s="35" t="n">
+      <x:c r="C40" s="43" t="n">
         <x:v>10000000</x:v>
       </x:c>
       <x:c r="D40" s="31" t="str">
@@ -55891,7 +56360,7 @@
       <x:c r="B41" s="31" t="str">
         <x:v>B39</x:v>
       </x:c>
-      <x:c r="C41" s="35" t="n">
+      <x:c r="C41" s="43" t="n">
         <x:v>7000000</x:v>
       </x:c>
       <x:c r="D41" s="31" t="str">
@@ -55911,7 +56380,7 @@
       <x:c r="B42" s="31" t="str">
         <x:v>B40</x:v>
       </x:c>
-      <x:c r="C42" s="35" t="n">
+      <x:c r="C42" s="43" t="n">
         <x:v>6000000</x:v>
       </x:c>
       <x:c r="D42" s="31" t="str">
@@ -55931,7 +56400,7 @@
       <x:c r="B43" s="31" t="str">
         <x:v>B42</x:v>
       </x:c>
-      <x:c r="C43" s="35" t="n">
+      <x:c r="C43" s="43" t="n">
         <x:v>15790000</x:v>
       </x:c>
       <x:c r="D43" s="31" t="str">
@@ -55951,7 +56420,7 @@
       <x:c r="B44" s="31" t="str">
         <x:v>D42</x:v>
       </x:c>
-      <x:c r="C44" s="35" t="n">
+      <x:c r="C44" s="43" t="n">
         <x:v>2137000</x:v>
       </x:c>
       <x:c r="D44" s="31" t="str">
@@ -55971,7 +56440,7 @@
       <x:c r="B45" s="31" t="str">
         <x:v>B43</x:v>
       </x:c>
-      <x:c r="C45" s="35" t="n">
+      <x:c r="C45" s="43" t="n">
         <x:v>700000</x:v>
       </x:c>
       <x:c r="D45" s="31" t="str">
@@ -55991,7 +56460,7 @@
       <x:c r="B46" s="31" t="str">
         <x:v>B45</x:v>
       </x:c>
-      <x:c r="C46" s="35" t="n">
+      <x:c r="C46" s="43" t="n">
         <x:v>23000000</x:v>
       </x:c>
       <x:c r="D46" s="31" t="str">
@@ -56011,7 +56480,7 @@
       <x:c r="B47" s="31" t="str">
         <x:v>D45</x:v>
       </x:c>
-      <x:c r="C47" s="35" t="n">
+      <x:c r="C47" s="43" t="n">
         <x:v>5000000</x:v>
       </x:c>
       <x:c r="D47" s="31" t="str">
@@ -56030,7 +56499,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rfdd9538190054bb5"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R8088b86e17384170"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -63397,24 +63866,94 @@
         <x:v>-5000000</x:v>
       </x:c>
     </x:row>
+    <x:row r="100" ht="24" hidden="0" customHeight="1">
+      <x:c r="A100" s="8" t="str">
+        <x:v>TX0096</x:v>
+      </x:c>
+      <x:c r="B100" s="9"/>
+      <x:c r="C100" s="8"/>
+      <x:c r="D100" s="8" t="str">
+        <x:v>Undated</x:v>
+      </x:c>
+      <x:c r="E100" s="8" t="str">
+        <x:v>Payment</x:v>
+      </x:c>
+      <x:c r="F100" s="11" t="n">
+        <x:v>3000000</x:v>
+      </x:c>
+      <x:c r="G100" s="12" t="str">
+        <x:v>toman</x:v>
+      </x:c>
+      <x:c r="H100" s="11" t="n">
+        <x:v>3000000</x:v>
+      </x:c>
+      <x:c r="I100" s="8" t="str">
+        <x:v>Domain registrar not supplied</x:v>
+      </x:c>
+      <x:c r="J100" s="31" t="str">
+        <x:v>Purchase of alenush.com for the association website; user-declared expense without receipt</x:v>
+      </x:c>
+      <x:c r="K100" s="31" t="str">
+        <x:v>خرید دامنهٔ alenush.com برای وب‌سایت انجمن؛ هزینهٔ اعلام‌شده توسط کاربر، بدون رسید</x:v>
+      </x:c>
+      <x:c r="L100" s="8" t="str">
+        <x:v>Website domain</x:v>
+      </x:c>
+      <x:c r="M100" s="8" t="str">
+        <x:v>Association website</x:v>
+      </x:c>
+      <x:c r="N100" s="8" t="str">
+        <x:v>Review</x:v>
+      </x:c>
+      <x:c r="O100" s="8" t="str">
+        <x:v>User declaration dated 2026-10-11; no receipt</x:v>
+      </x:c>
+      <x:c r="P100" s="8" t="str">
+        <x:v>Unknown funding source</x:v>
+      </x:c>
+      <x:c r="Q100" s="8" t="str"/>
+      <x:c r="R100" s="8"/>
+      <x:c r="S100" s="8"/>
+      <x:c r="T100" s="31" t="str">
+        <x:v>Purpose and reported purchase amount confirmed by user. Purchase date, funding source and any reimbursement are unknown; not yet included in the cutoff cash totals.</x:v>
+      </x:c>
+      <x:c r="U100" s="31" t="str">
+        <x:v>The VM creation date is not used as the domain purchase date. Keep the declared domain expense separate from confirmed association cash disbursements until date and funding are clarified.</x:v>
+      </x:c>
+      <x:c r="V100" s="31" t="str">
+        <x:v>reports/2026-10-10/website_user_confirmation_2026-10-11.json</x:v>
+      </x:c>
+      <x:c r="W100" s="13" t="n">
+        <x:f>IF(AND(N100="Supported",E100="Receipt",ISNUMBER(H100)),H100,0)</x:f>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="X100" s="13" t="n">
+        <x:f>IF(AND(N100="Supported",E100="Payment",ISNUMBER(H100)),H100,0)</x:f>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="Y100" s="13" t="n">
+        <x:f>W100-X100</x:f>
+        <x:v>0</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:mergeCells>
     <x:mergeCell ref="A2:F2"/>
   </x:mergeCells>
-  <x:conditionalFormatting sqref="N5:N99">
+  <x:conditionalFormatting sqref="N5:N100">
     <x:cfRule type="containsText" dxfId="0" priority="1" operator="containsText" text="Review"/>
   </x:conditionalFormatting>
   <x:dataValidations count="2">
-    <x:dataValidation type="list" sqref="N5:N99">
+    <x:dataValidation type="list" sqref="N5:N100">
       <x:formula1>"Supported,Review,Duplicate,Invoice only,Summary only"</x:formula1>
     </x:dataValidation>
-    <x:dataValidation type="list" sqref="E5:E99">
+    <x:dataValidation type="list" sqref="E5:E100">
       <x:formula1>"Receipt,Payment,Internal transfer,Unknown"</x:formula1>
     </x:dataValidation>
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R42ab8608d7634931"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R4306b05e5e124627"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -63440,45 +63979,45 @@
   </x:cols>
   <x:sheetData>
     <x:row r="1" ht="15" hidden="0" customHeight="1">
-      <x:c r="A1" s="33"/>
-      <x:c r="B1" s="33"/>
-      <x:c r="C1" s="33"/>
-      <x:c r="D1" s="33"/>
-      <x:c r="E1" s="33"/>
-      <x:c r="F1" s="33"/>
-      <x:c r="G1" s="33"/>
-      <x:c r="H1" s="33"/>
-      <x:c r="I1" s="33"/>
-      <x:c r="J1" s="33"/>
-      <x:c r="K1" s="33"/>
+      <x:c r="A1" s="39"/>
+      <x:c r="B1" s="39"/>
+      <x:c r="C1" s="39"/>
+      <x:c r="D1" s="39"/>
+      <x:c r="E1" s="39"/>
+      <x:c r="F1" s="39"/>
+      <x:c r="G1" s="39"/>
+      <x:c r="H1" s="39"/>
+      <x:c r="I1" s="39"/>
+      <x:c r="J1" s="39"/>
+      <x:c r="K1" s="39"/>
     </x:row>
     <x:row r="2" ht="16.799999237060547" hidden="0" customHeight="1">
-      <x:c r="A2" s="34" t="str">
+      <x:c r="A2" s="40" t="str">
         <x:v>Supplier invoice and payment matching register</x:v>
       </x:c>
-      <x:c r="B2" s="33"/>
-      <x:c r="C2" s="33"/>
-      <x:c r="D2" s="33"/>
-      <x:c r="E2" s="33"/>
-      <x:c r="F2" s="33"/>
-      <x:c r="G2" s="33"/>
-      <x:c r="H2" s="33"/>
-      <x:c r="I2" s="33"/>
-      <x:c r="J2" s="33"/>
-      <x:c r="K2" s="33"/>
+      <x:c r="B2" s="39"/>
+      <x:c r="C2" s="39"/>
+      <x:c r="D2" s="39"/>
+      <x:c r="E2" s="39"/>
+      <x:c r="F2" s="39"/>
+      <x:c r="G2" s="39"/>
+      <x:c r="H2" s="39"/>
+      <x:c r="I2" s="39"/>
+      <x:c r="J2" s="39"/>
+      <x:c r="K2" s="39"/>
     </x:row>
     <x:row r="3" ht="15" hidden="0" customHeight="1">
-      <x:c r="A3" s="33"/>
-      <x:c r="B3" s="33"/>
-      <x:c r="C3" s="33"/>
-      <x:c r="D3" s="33"/>
-      <x:c r="E3" s="33"/>
-      <x:c r="F3" s="33"/>
-      <x:c r="G3" s="33"/>
-      <x:c r="H3" s="33"/>
-      <x:c r="I3" s="33"/>
-      <x:c r="J3" s="33"/>
-      <x:c r="K3" s="33"/>
+      <x:c r="A3" s="39"/>
+      <x:c r="B3" s="39"/>
+      <x:c r="C3" s="39"/>
+      <x:c r="D3" s="39"/>
+      <x:c r="E3" s="39"/>
+      <x:c r="F3" s="39"/>
+      <x:c r="G3" s="39"/>
+      <x:c r="H3" s="39"/>
+      <x:c r="I3" s="39"/>
+      <x:c r="J3" s="39"/>
+      <x:c r="K3" s="39"/>
     </x:row>
     <x:row r="4" ht="15" hidden="0" customHeight="1">
       <x:c r="A4" s="7" t="str">
@@ -63529,10 +64068,10 @@
         <x:v>Sony NP-FV50 battery, invoice 15628595</x:v>
       </x:c>
       <x:c r="E5" s="31"/>
-      <x:c r="F5" s="35" t="n">
+      <x:c r="F5" s="43" t="n">
         <x:v>696000</x:v>
       </x:c>
-      <x:c r="G5" s="35" t="n">
+      <x:c r="G5" s="43" t="n">
         <x:v>0</x:v>
       </x:c>
       <x:c r="H5" s="31" t="str">
@@ -63562,10 +64101,10 @@
         <x:v>Shipping and insurance, invoice 12050044</x:v>
       </x:c>
       <x:c r="E6" s="31"/>
-      <x:c r="F6" s="35" t="n">
+      <x:c r="F6" s="43" t="n">
         <x:v>29000</x:v>
       </x:c>
-      <x:c r="G6" s="35" t="n">
+      <x:c r="G6" s="43" t="n">
         <x:v>0</x:v>
       </x:c>
       <x:c r="H6" s="31" t="str">
@@ -63595,10 +64134,10 @@
         <x:v>4 balloon glue, invoice 29449</x:v>
       </x:c>
       <x:c r="E7" s="31"/>
-      <x:c r="F7" s="35" t="n">
+      <x:c r="F7" s="43" t="n">
         <x:v>120000</x:v>
       </x:c>
-      <x:c r="G7" s="35"/>
+      <x:c r="G7" s="43"/>
       <x:c r="H7" s="31" t="str">
         <x:v>TX0037</x:v>
       </x:c>
@@ -63627,10 +64166,10 @@
         <x:v>Balloons, pump, thread, foils; invoice 2935/29350</x:v>
       </x:c>
       <x:c r="E8" s="31"/>
-      <x:c r="F8" s="35" t="n">
+      <x:c r="F8" s="43" t="n">
         <x:v>1310000</x:v>
       </x:c>
-      <x:c r="G8" s="35"/>
+      <x:c r="G8" s="43"/>
       <x:c r="H8" s="31" t="str">
         <x:v>TX0038</x:v>
       </x:c>
@@ -63657,8 +64196,8 @@
         <x:v>Freshman prizes: holders, spinners, bow ties</x:v>
       </x:c>
       <x:c r="E9" s="31"/>
-      <x:c r="F9" s="35"/>
-      <x:c r="G9" s="35"/>
+      <x:c r="F9" s="43"/>
+      <x:c r="G9" s="43"/>
       <x:c r="H9" s="31" t="str">
         <x:v>TX0033</x:v>
       </x:c>
@@ -63686,10 +64225,10 @@
         <x:v>USB flash 32G and earphones</x:v>
       </x:c>
       <x:c r="E10" s="31"/>
-      <x:c r="F10" s="35" t="n">
+      <x:c r="F10" s="43" t="n">
         <x:v>1500000</x:v>
       </x:c>
-      <x:c r="G10" s="35"/>
+      <x:c r="G10" s="43"/>
       <x:c r="H10" s="31" t="str">
         <x:v>TX0034</x:v>
       </x:c>
@@ -63717,10 +64256,10 @@
         <x:v>Pineapple pie and pastry order</x:v>
       </x:c>
       <x:c r="E11" s="31"/>
-      <x:c r="F11" s="35" t="n">
+      <x:c r="F11" s="43" t="n">
         <x:v>1052375</x:v>
       </x:c>
-      <x:c r="G11" s="35"/>
+      <x:c r="G11" s="43"/>
       <x:c r="H11" s="31" t="str">
         <x:v>TX0024</x:v>
       </x:c>
@@ -63748,10 +64287,10 @@
         <x:v>French chocolate cream pastry</x:v>
       </x:c>
       <x:c r="E12" s="31"/>
-      <x:c r="F12" s="35" t="n">
+      <x:c r="F12" s="43" t="n">
         <x:v>912850</x:v>
       </x:c>
-      <x:c r="G12" s="35"/>
+      <x:c r="G12" s="43"/>
       <x:c r="H12" s="31" t="str">
         <x:v>TX0023</x:v>
       </x:c>
@@ -63777,10 +64316,10 @@
         <x:v>7 × 2kg pomegranates</x:v>
       </x:c>
       <x:c r="E13" s="31"/>
-      <x:c r="F13" s="35" t="n">
+      <x:c r="F13" s="43" t="n">
         <x:v>1664700</x:v>
       </x:c>
-      <x:c r="G13" s="35"/>
+      <x:c r="G13" s="43"/>
       <x:c r="H13" s="31" t="str"/>
       <x:c r="I13" s="31" t="str">
         <x:v>Unmatched invoice</x:v>
@@ -63806,10 +64345,10 @@
         <x:v>Jelly powder and cherry syrup</x:v>
       </x:c>
       <x:c r="E14" s="31"/>
-      <x:c r="F14" s="35" t="n">
+      <x:c r="F14" s="43" t="n">
         <x:v>2150000</x:v>
       </x:c>
-      <x:c r="G14" s="35" t="n">
+      <x:c r="G14" s="43" t="n">
         <x:v>195454.5</x:v>
       </x:c>
       <x:c r="H14" s="31" t="str">
@@ -63840,10 +64379,10 @@
         <x:v>Snack receipts C1-C8 (eight slips)</x:v>
       </x:c>
       <x:c r="E15" s="31"/>
-      <x:c r="F15" s="35" t="n">
+      <x:c r="F15" s="43" t="n">
         <x:v>1306700</x:v>
       </x:c>
-      <x:c r="G15" s="35"/>
+      <x:c r="G15" s="43"/>
       <x:c r="H15" s="31" t="str">
         <x:v>TX0064, TX0065, TX0066, TX0067, TX0068, TX0069, TX0072, TX0073</x:v>
       </x:c>
@@ -63871,10 +64410,10 @@
         <x:v>99 Mozmoz snacks</x:v>
       </x:c>
       <x:c r="E16" s="31"/>
-      <x:c r="F16" s="35" t="n">
+      <x:c r="F16" s="43" t="n">
         <x:v>1916640</x:v>
       </x:c>
-      <x:c r="G16" s="35" t="n">
+      <x:c r="G16" s="43" t="n">
         <x:v>174240</x:v>
       </x:c>
       <x:c r="H16" s="31" t="str">
@@ -63904,10 +64443,10 @@
         <x:v>Gala chocolate</x:v>
       </x:c>
       <x:c r="E17" s="31"/>
-      <x:c r="F17" s="35" t="n">
+      <x:c r="F17" s="43" t="n">
         <x:v>135800</x:v>
       </x:c>
-      <x:c r="G17" s="35" t="n">
+      <x:c r="G17" s="43" t="n">
         <x:v>12345.4</x:v>
       </x:c>
       <x:c r="H17" s="31" t="str">
@@ -63935,10 +64474,10 @@
         <x:v>Handwritten, likely chocolate cookies</x:v>
       </x:c>
       <x:c r="E18" s="31"/>
-      <x:c r="F18" s="35" t="n">
+      <x:c r="F18" s="43" t="n">
         <x:v>495000</x:v>
       </x:c>
-      <x:c r="G18" s="35"/>
+      <x:c r="G18" s="43"/>
       <x:c r="H18" s="31" t="str"/>
       <x:c r="I18" s="31" t="str">
         <x:v>Unmatched invoice</x:v>
@@ -63964,10 +64503,10 @@
         <x:v>Skyroom licence + recording, invoice 61150</x:v>
       </x:c>
       <x:c r="E19" s="31"/>
-      <x:c r="F19" s="35" t="n">
+      <x:c r="F19" s="43" t="n">
         <x:v>4257000</x:v>
       </x:c>
-      <x:c r="G19" s="35" t="n">
+      <x:c r="G19" s="43" t="n">
         <x:v>387000</x:v>
       </x:c>
       <x:c r="H19" s="31" t="str"/>
@@ -63995,10 +64534,10 @@
         <x:v>190 dairy drinks and cakes, order 165826</x:v>
       </x:c>
       <x:c r="E20" s="31"/>
-      <x:c r="F20" s="35" t="n">
+      <x:c r="F20" s="43" t="n">
         <x:v>9987900</x:v>
       </x:c>
-      <x:c r="G20" s="35"/>
+      <x:c r="G20" s="43"/>
       <x:c r="H20" s="31" t="str">
         <x:v>TX0089</x:v>
       </x:c>
@@ -64019,7 +64558,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R44849797a5ce4847"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rfb42093059a64c5e"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -64042,36 +64581,36 @@
   </x:cols>
   <x:sheetData>
     <x:row r="1" ht="15" hidden="0" customHeight="1">
-      <x:c r="A1" s="33"/>
-      <x:c r="B1" s="33"/>
-      <x:c r="C1" s="33"/>
-      <x:c r="D1" s="33"/>
-      <x:c r="E1" s="33"/>
-      <x:c r="F1" s="33"/>
-      <x:c r="G1" s="33"/>
-      <x:c r="H1" s="33"/>
+      <x:c r="A1" s="39"/>
+      <x:c r="B1" s="39"/>
+      <x:c r="C1" s="39"/>
+      <x:c r="D1" s="39"/>
+      <x:c r="E1" s="39"/>
+      <x:c r="F1" s="39"/>
+      <x:c r="G1" s="39"/>
+      <x:c r="H1" s="39"/>
     </x:row>
     <x:row r="2" ht="16.799999237060547" hidden="0" customHeight="1">
-      <x:c r="A2" s="34" t="str">
+      <x:c r="A2" s="40" t="str">
         <x:v>Reconciliation issues and required follow-up</x:v>
       </x:c>
-      <x:c r="B2" s="33"/>
-      <x:c r="C2" s="33"/>
-      <x:c r="D2" s="33"/>
-      <x:c r="E2" s="33"/>
-      <x:c r="F2" s="33"/>
-      <x:c r="G2" s="33"/>
-      <x:c r="H2" s="33"/>
+      <x:c r="B2" s="39"/>
+      <x:c r="C2" s="39"/>
+      <x:c r="D2" s="39"/>
+      <x:c r="E2" s="39"/>
+      <x:c r="F2" s="39"/>
+      <x:c r="G2" s="39"/>
+      <x:c r="H2" s="39"/>
     </x:row>
     <x:row r="3" ht="15" hidden="0" customHeight="1">
-      <x:c r="A3" s="33"/>
-      <x:c r="B3" s="33"/>
-      <x:c r="C3" s="33"/>
-      <x:c r="D3" s="33"/>
-      <x:c r="E3" s="33"/>
-      <x:c r="F3" s="33"/>
-      <x:c r="G3" s="33"/>
-      <x:c r="H3" s="33"/>
+      <x:c r="A3" s="39"/>
+      <x:c r="B3" s="39"/>
+      <x:c r="C3" s="39"/>
+      <x:c r="D3" s="39"/>
+      <x:c r="E3" s="39"/>
+      <x:c r="F3" s="39"/>
+      <x:c r="G3" s="39"/>
+      <x:c r="H3" s="39"/>
     </x:row>
     <x:row r="4" ht="15" hidden="0" customHeight="1">
       <x:c r="A4" s="7" t="str">
@@ -64112,7 +64651,7 @@
       <x:c r="D5" s="31" t="str">
         <x:v>Only fragments are available: receipts, SMS and screenshots. There is no opening balance, and balance snapshots conflict (230,203,965 rial on 1404/05/02; 22,953,913 rial on 1404/07/20; '560,800,163' on 1404/07/22; 22,765,000 in message52; 29,200 in message86). The 560,800,163 and 565,800,163 rial snapshots are mutually consistent with a 5,000,000 rial deposit; their relation to the earlier 22,953,913 snapshot remains unexplained. On 1404/05/03 the balance drop of 9,614,400 rial is 7,394,600 smaller than recorded intervening debits of 17,009,000 rial, requiring inflows or other explanation.</x:v>
       </x:c>
-      <x:c r="E5" s="35"/>
+      <x:c r="E5" s="43"/>
       <x:c r="F5" s="31" t="str"/>
       <x:c r="G5" s="31" t="str">
         <x:v>Obtain full Shahr 400816808774, Sepah 3001254062925 and Blu statements.</x:v>
@@ -64134,7 +64673,7 @@
       <x:c r="D6" s="31" t="str">
         <x:v>User confirms all eleven Blu outflows totaling 33,937,250 are association expenses. Five identified Summer School 1405 fees total 11,500,000; sticker packs cost 950,000. Remaining 21,487,250 requires purpose/project allocation, not income/expense-direction confirmation.</x:v>
       </x:c>
-      <x:c r="E6" s="35" t="n">
+      <x:c r="E6" s="43" t="n">
         <x:v>33937250</x:v>
       </x:c>
       <x:c r="F6" s="31" t="str">
@@ -64160,7 +64699,7 @@
       <x:c r="D7" s="31" t="str">
         <x:v>User confirms seven Shahr-folder outflows totaling 14,038,220 are association expenses, including TX0061 previously unclassified in direction. Merchant/project allocation remains pending. The unlogged balance movement remains unexplained.</x:v>
       </x:c>
-      <x:c r="E7" s="35" t="n">
+      <x:c r="E7" s="43" t="n">
         <x:v>14038220</x:v>
       </x:c>
       <x:c r="F7" s="31" t="str">
@@ -64186,7 +64725,7 @@
       <x:c r="D8" s="31" t="str">
         <x:v>Platform gross sales 27,235,000 vs original-ledger receipts 23,000,000 remain unreconciled. Skyroom invoice 4,257,000 remains unmatched. Food invoice 9,987,900 is now user-confirmed paid (TX0089); sticker purchase 950,000 belongs to this event (TX0088). No new registration receipts are inferred.</x:v>
       </x:c>
-      <x:c r="E8" s="35" t="n">
+      <x:c r="E8" s="43" t="n">
         <x:v>4235000</x:v>
       </x:c>
       <x:c r="F8" s="31" t="str">
@@ -64213,7 +64752,7 @@
       <x:c r="D9" s="31" t="str">
         <x:v>17,650,000 without a unit. As rial (1,765,000 toman) it equals ledger M3 net. Treated as an internal transfer.</x:v>
       </x:c>
-      <x:c r="E9" s="35"/>
+      <x:c r="E9" s="43"/>
       <x:c r="F9" s="31" t="str">
         <x:v>TX0018, TX0014</x:v>
       </x:c>
@@ -64237,7 +64776,7 @@
       <x:c r="D10" s="31" t="str">
         <x:v>مجموع D23 duplicates the D20 pastry (1,052,375). D12 likely duplicates the D9 ad (400,000).</x:v>
       </x:c>
-      <x:c r="E10" s="35" t="n">
+      <x:c r="E10" s="43" t="n">
         <x:v>1452375</x:v>
       </x:c>
       <x:c r="F10" s="31" t="str">
@@ -64264,7 +64803,7 @@
       <x:c r="D11" s="31" t="str">
         <x:v>message111 reads '300000 cash shabash for the party'. The ledger treats it as an expense (D29), but it could be cash received. This Telegram/workbook item is outside recipts/ and is not resolved by the folder-wide expense confirmation.</x:v>
       </x:c>
-      <x:c r="E11" s="35" t="n">
+      <x:c r="E11" s="43" t="n">
         <x:v>300000</x:v>
       </x:c>
       <x:c r="F11" s="31" t="str">
@@ -64290,7 +64829,7 @@
       <x:c r="D12" s="31" t="str">
         <x:v>Parnian reimbursement 4,050,000 is absent from the original ledger. Printed purchases total 3,359,139.9, or 3,180,139.9 excluding possible C6 duplicate. Including invoice-only Ribar 495,000 gives 3,854,139.9 or 3,675,139.9. These are provisional documentation gaps, not confirmed overpayment. Hossein reimbursement is undocumented. Bardia claims vs payment need a separate bridge.</x:v>
       </x:c>
-      <x:c r="E12" s="35" t="n">
+      <x:c r="E12" s="43" t="n">
         <x:v>4050000</x:v>
       </x:c>
       <x:c r="F12" s="31" t="str">
@@ -64316,7 +64855,7 @@
       <x:c r="D13" s="31" t="str">
         <x:v>The SMS withdrawal is 100,037,800 in an unprinted unit (10,003,780 toman if rial). Message120 describes expense payments or transfers, not income. It remains unconverted and may overlap recorded expenses. Deposit lines are explicitly rial: 150,000, 500,000 and 1,000,000 toman; they do not sum to the treasurer total 15,790,000. Balances imply unlogged movements.</x:v>
       </x:c>
-      <x:c r="E13" s="35"/>
+      <x:c r="E13" s="43"/>
       <x:c r="F13" s="31" t="str">
         <x:v>TX0049, TX0047</x:v>
       </x:c>
@@ -64340,7 +64879,7 @@
       <x:c r="D14" s="31" t="str">
         <x:v>The receipt shows 235,000; the ledger and message show 230,000.</x:v>
       </x:c>
-      <x:c r="E14" s="35" t="n">
+      <x:c r="E14" s="43" t="n">
         <x:v>5000</x:v>
       </x:c>
       <x:c r="F14" s="31" t="str">
@@ -64366,7 +64905,7 @@
       <x:c r="D15" s="31" t="str">
         <x:v>Transfer fee 900, Dina Zali 180,000, Parnian 4,050,000. The poster print of 13,000 is unmatched.</x:v>
       </x:c>
-      <x:c r="E15" s="35" t="n">
+      <x:c r="E15" s="43" t="n">
         <x:v>4230900</x:v>
       </x:c>
       <x:c r="F15" s="31" t="str">
@@ -64390,7 +64929,7 @@
       <x:c r="D16" s="31" t="str">
         <x:v>Refined تطبیق!B7 is circular (=B6-B7; should be B5-B6). TX-00002 counterparty is wrong. TX-00044 is marked confirmed with no payment. The مرداد sheet omits D10-D12. Sohrab's fee does not follow the 100k rounding rule (2,934→3,000).</x:v>
       </x:c>
-      <x:c r="E16" s="35"/>
+      <x:c r="E16" s="43"/>
       <x:c r="F16" s="31" t="str">
         <x:v>TX0001, TX0002, TX0082</x:v>
       </x:c>
@@ -64414,7 +64953,7 @@
       <x:c r="D17" s="31" t="str">
         <x:v>Moghimi's 10m receipt has no date. The forward header is 1404/08/28 but the ledger month is آذر.</x:v>
       </x:c>
-      <x:c r="E17" s="35" t="n">
+      <x:c r="E17" s="43" t="n">
         <x:v>10000000</x:v>
       </x:c>
       <x:c r="F17" s="31" t="str">
@@ -64440,7 +64979,7 @@
       <x:c r="D18" s="31" t="str">
         <x:v>Course reports label 11,601, 12,261 and 9,781 as toman. The printed-unit total is 33,643 toman. A possible thousand-toman scale would total 33,643,000, versus the ledger 33,642,000; that scale is unconfirmed and is used only as a comparison, not additional revenue. Reports contain student phone numbers.</x:v>
       </x:c>
-      <x:c r="E18" s="35" t="n">
+      <x:c r="E18" s="43" t="n">
         <x:v>1000</x:v>
       </x:c>
       <x:c r="F18" s="31" t="str">
@@ -64466,7 +65005,7 @@
       <x:c r="D19" s="31" t="str">
         <x:v>User states six folder receipts are instructor payments. Five are matched by recipient-name evidence and explicit clarification: TX0083-87, total 11,500,000. TX0088 is explicitly sticker packs, not an instructor fee. The sixth remains unmatched among already recorded folder expenses.</x:v>
       </x:c>
-      <x:c r="E19" s="35"/>
+      <x:c r="E19" s="43"/>
       <x:c r="F19" s="31" t="str">
         <x:v>TX0083, TX0084, TX0085, TX0086, TX0087</x:v>
       </x:c>
@@ -64475,6 +65014,32 @@
       </x:c>
       <x:c r="H19" s="31" t="str">
         <x:v>reports/2026-10-10/user_confirmation_2026-10-10.json</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="20" ht="24" hidden="0" customHeight="1">
+      <x:c r="A20" s="31" t="str">
+        <x:v>ISS016</x:v>
+      </x:c>
+      <x:c r="B20" s="31" t="str">
+        <x:v>Medium</x:v>
+      </x:c>
+      <x:c r="C20" s="31" t="str">
+        <x:v>Website domain payment date and funding source</x:v>
+      </x:c>
+      <x:c r="D20" s="31" t="str">
+        <x:v>User reports paying 3,000,000 toman for alenush.com, without a designated receipt. Association purpose is confirmed. The purchase date and whether association or personal funds paid it are unknown. Actual VM payments are also not supplied; the 92-day VM figure is a budget estimate.</x:v>
+      </x:c>
+      <x:c r="E20" s="43" t="n">
+        <x:v>3000000</x:v>
+      </x:c>
+      <x:c r="F20" s="31" t="str">
+        <x:v>TX0096</x:v>
+      </x:c>
+      <x:c r="G20" s="31" t="str">
+        <x:v>Record the purchase date and funding account; identify any reimbursement and obtain registrar confirmation if available. Replace VM estimates with actual billing records when supplied.</x:v>
+      </x:c>
+      <x:c r="H20" s="31" t="str">
+        <x:v>reports/2026-10-10/website_user_confirmation_2026-10-11.json</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -64483,7 +65048,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rc9cbf4759baa4eb2"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R5621255d72c24ad2"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>